<commit_message>
docs: include exact skill scaling curves and simplify SP cost display
Replace generic skill descriptions with exact effect and level-up values from QoL dataset. Replace complex SP parentheses with clean Total SP column.
</commit_message>
<xml_diff>
--- a/data_tables/guide_text.xlsx
+++ b/data_tables/guide_text.xlsx
@@ -498,7 +498,6 @@
           <t>#### Stat Growth</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -528,7 +527,6 @@
           <t>#### Class Overview</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -592,7 +590,6 @@
           <t>#### Learned Skills</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -918,7 +915,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Effect &amp; Scaling</t>
         </is>
       </c>
     </row>
@@ -1110,7 +1107,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>SP Cost</t>
+          <t>Total SP</t>
         </is>
       </c>
     </row>
@@ -2953,7 +2950,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D313"/>
+  <dimension ref="A1:E313"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2977,6 +2974,11 @@
           <t>Description</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Scaling</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2997,6 +2999,12 @@
           <t>Attract an enemy's attacks.</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Enmity: 250
+Turns: 3 -&gt; 4 -&gt; 5 -&gt; 6 -&gt; 7   |   TP Cost: 1 -&gt; 2 -&gt; 3 -&gt; 4 -&gt; 5   |   Speed: 1.5x -&gt; 2x</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3017,6 +3025,12 @@
           <t>Attract all enemies' attacks.</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Enmity: 150
+Turns: 3 -&gt; 4 -&gt; 5 -&gt; 6 -&gt; 7 | TP Cost: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 | Speed: 1.25x -&gt; 1.77x</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3037,6 +3051,12 @@
           <t>Raise the party's ATK.</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>ATK: +8% -&gt; +10% -&gt; +12% -&gt; +15% -&gt; +18% (L1-5 Max)
+Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8   |   TP Cost: 5 -&gt; 7 -&gt; 9 -&gt; 11 -&gt; 13</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3057,6 +3077,12 @@
           <t>Short-range skill. Powerful strike to one enemy.</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>ATK: 125% -&gt; 134 -&gt; 143 -&gt; 152 -&gt; 161 -&gt; 170 -&gt; 178 -&gt; 186 -&gt; 193 -&gt; 200% (L10)
+Accuracy: +20% (+2%/Lv)   |   TP Cost: 5 (+2-3/Lv) -&gt; 28   |   Speed: 0.8x -&gt; 0.9x</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3077,6 +3103,12 @@
           <t>Short-range skill. Attack one enemy. May cancel enemy buffs.</t>
         </is>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Accuracy: +20% -&gt; +22 -&gt; +24 -&gt; +26 -&gt; +28 -&gt; +30 -&gt; +31 -&gt; +32 -&gt; +33 -&gt; +35% (L10)
+Buff cancel rate: 68% (+1-2%/Lv) -&gt; 85%   |   TP Cost: 5 (+1-2/Lv) -&gt; 18   |   Speed: 0.9x</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3097,6 +3129,12 @@
           <t>Increase own ATK at the price of lowering own DEF.</t>
         </is>
       </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>ATK: +20% -&gt; +30% -&gt; +40% -&gt; +45% -&gt; +50% (L1-5 Max)
+DEF: -11% -&gt; -14% -&gt; -17% -&gt; -21% -&gt; -25%   |   Turns: 4 -&gt; 8   |   TP Cost: 8 (+2/Lv) -&gt; 16</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3117,6 +3155,12 @@
           <t>Increase own DEF at the price of lowering own ATK.</t>
         </is>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>DEF: +20% -&gt; +30% -&gt; +40% -&gt; +45% -&gt; +50% (L1-5 Max)
+ATK: -11% -&gt; -14% -&gt; -17% -&gt; -21% -&gt; -25%   |   Turns: 4 -&gt; 8   |   TP Cost: 8 (+2/Lv) -&gt; 16</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3137,6 +3181,12 @@
           <t>Shield skill. Deal bash damage to one enemy. May stun.</t>
         </is>
       </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>ATK: 85% -&gt; 90% -&gt; 94% -&gt; 98% -&gt; 102% (L1-5 Max)   |   Accuracy: +6% (+3-4%/Lv) -&gt; +20%
+Stun: 30% -&gt; 32% -&gt; 34% -&gt; 36% -&gt; 38%   |   TP Cost: 6 -&gt; 8 -&gt; 10 -&gt; 12 -&gt; 14</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3157,6 +3207,12 @@
           <t>Katana skill. Deal bash damage to one enemy. May paralyze.</t>
         </is>
       </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>ATK: 106% -&gt; 112 -&gt; 118 -&gt; 124 -&gt; 130 -&gt; 134 -&gt; 138 -&gt; 142 -&gt; 146 -&gt; 150% (L10)
+Accuracy: +5% (+2-3%/Lv) -&gt; +28%   |   Paralysis: 20% -&gt; 50%   |   TP Cost: 6 (+2/Lv) -&gt; 24</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3177,6 +3233,12 @@
           <t>Raise own critical rate, but also own vulnerability to critical hits.</t>
         </is>
       </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Critical rate: 5% (+2.5%/Lv) -&gt; 15% (L5 Max)   |   Enemy critical rate: 4% (+2%/Lv)
+Turns: 6 -&gt; 7 -&gt; 8 -&gt; 9 -&gt; 10   |   TP Cost: 12 -&gt; 14 -&gt; 16 -&gt; 18 -&gt; 20</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3197,6 +3259,12 @@
           <t>Katana skill. Deal slash damage to an enemy row. May instakill.</t>
         </is>
       </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>ATK: 80% -&gt; 83 -&gt; 86 -&gt; 89 -&gt; 91 -&gt; 94 -&gt; 97 -&gt; 100 -&gt; 105 -&gt; 110% (L10)
+Instakill: 10% (+1-2%/Lv) -&gt; 20%   |   Power decrease: 10%   |   TP Cost: 38 (+4/Lv) -&gt; 74</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3217,6 +3285,12 @@
           <t>Katana skill. Deal defense-piercing damage and DEF down to one enemy.</t>
         </is>
       </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>ATK: 84% -&gt; 88 -&gt; 92 -&gt; 96 -&gt; 100 -&gt; 104 -&gt; 108 -&gt; 112 -&gt; 116 -&gt; 120% (L10)
+Enemy DEF: -16% (-1%/Lv)   |   Turns: 4   |   TP Cost: 14 (+2/Lv) -&gt; 32   |   Speed: 0.8x</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3237,6 +3311,12 @@
           <t>Katana skill. Deal slash damage to an enemy row.</t>
         </is>
       </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>ATK: 104% -&gt; 108 -&gt; 112 -&gt; 116 -&gt; 120 -&gt; 124 -&gt; 128 -&gt; 132 -&gt; 136 -&gt; 140% (L10)
+TP Cost: 22 -&gt; 26 -&gt; 30 -&gt; 34 -&gt; 38 -&gt; 42 -&gt; 46 -&gt; 50 -&gt; 54 -&gt; 58</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3257,6 +3337,12 @@
           <t>Katana skill. Deal slash damage 3 times to one enemy. Living targets only.</t>
         </is>
       </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>ATK: 118% -&gt; 120 -&gt; 124 -&gt; 128 -&gt; 132 -&gt; 136 -&gt; 140 -&gt; 146 -&gt; 152 -&gt; 158% (L10)
+Critical rate: 10%   |   TP Cost: 36 (+2-3/Lv) -&gt; 61   |   Speed: 0.7x -&gt; 0.8x</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3277,6 +3363,12 @@
           <t>Short-range skill. Attack one enemy to regain HP.</t>
         </is>
       </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>ATK: 74% (+4%/Lv) -&gt; 110% (L10 Max)   |   HP Absorb: 15% (+1-2%/Lv) -&gt; 25%
+TP Cost: 12 -&gt; 15 -&gt; 18 -&gt; 21 -&gt; 24 -&gt; 27 -&gt; 30 -&gt; 32 -&gt; 34 -&gt; 36   |   Speed: 0.9x</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3297,6 +3389,12 @@
           <t>Short-range skill. Attack one enemy to regain TP.</t>
         </is>
       </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>ATK: 65% -&gt; 70 -&gt; 75 -&gt; 80 -&gt; 84 -&gt; 88 -&gt; 91 -&gt; 94 -&gt; 97 -&gt; 100% (L10)
+TP Absorb: 10% (+1-2%/Lv) -&gt; 20%   |   TP Cost: 6 (+2/Lv) -&gt; 24   |   Speed: 0.9x</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3317,6 +3415,12 @@
           <t>Short-range skill. Deal mid-range water damage to one enemy. May freeze.</t>
         </is>
       </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>ATK: 130% -&gt; 144 -&gt; 157 -&gt; 170 -&gt; 182 -&gt; 194 -&gt; 204 -&gt; 212 -&gt; 220 -&gt; 228% (L10)
+Freeze: 20% (+3-4%/Lv) -&gt; 50%   |   Accuracy: +14%   |   TP Cost: 9 (+3/Lv) -&gt; 36</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3337,6 +3441,12 @@
           <t>Axe skill. Deal earth damage to one enemy. May petrify.</t>
         </is>
       </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>ATK: 135% (+11-14%/Lv) -&gt; 247%   |   Petrify: 20% (+1-2%/Lv) -&gt; 35%   |   Accuracy: +10%
+TP Cost: 9 -&gt; 12 -&gt; 15 -&gt; 18 -&gt; 21 -&gt; 24 -&gt; 28 -&gt; 32 -&gt; 37 -&gt; 42</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3357,6 +3467,12 @@
           <t>Axe skill. Attack an enemy, then the next immediate enemy in the turn order.</t>
         </is>
       </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>ATK: 120% -&gt; 130 -&gt; 140 -&gt; 148 -&gt; 156 -&gt; 164 -&gt; 170 -&gt; 176 -&gt; 180 -&gt; 184% (L10)
+Targets: 2 (Lv1-3) -&gt; 3 (Lv4-6) -&gt; 4 (Lv7-8) -&gt; 5 (L9-10)   |   TP: 26 (+4-6/Lv) -&gt; 68</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3377,6 +3493,12 @@
           <t>Take all physical damage in place of one ally.</t>
         </is>
       </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Cover ends per hit: 70% -&gt; 62% -&gt; 54% -&gt; 46% -&gt; 40% (L1-5 Max)
+Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8   |   TP Cost: 10 -&gt; 14 -&gt; 18 -&gt; 21 -&gt; 24</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3397,6 +3519,12 @@
           <t>Short-range skill. Use one's weapon to repel enemy attacks.</t>
         </is>
       </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Parry ends per block: 80% -&gt; 72% -&gt; 64% -&gt; 58% -&gt; 52% (L1-5 Max)
+Turns: 3 -&gt; 4 -&gt; 5 -&gt; 6 -&gt; 7   |   TP Cost: 14 -&gt; 17 -&gt; 20 -&gt; 23 -&gt; 26</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3417,6 +3545,12 @@
           <t>Sword/lance skill. Attack one enemy (effective vs. unholy monsters).</t>
         </is>
       </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>ATK: 130% -&gt; 140 -&gt; 150 -&gt; 160 -&gt; 170 -&gt; 180 -&gt; 190 -&gt; 200 -&gt; 211 -&gt; 222% (L10)
+Accuracy: +6% -&gt; +20%   |   Damage vs. unholy: +65%   |   TP Cost: 12 (+3/Lv) -&gt; 39</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3437,6 +3571,12 @@
           <t>Shield skill. Reduce physical damage taken by the party once.</t>
         </is>
       </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Damage reduction rate: 12% -&gt; 14 -&gt; 16 -&gt; 18 -&gt; 20 -&gt; 22 -&gt; 24 -&gt; 26 -&gt; 28 -&gt; 30%
+Turns: 5   |   TP Cost: 20 -&gt; 23 -&gt; 26 -&gt; 29 -&gt; 31 -&gt; 34 -&gt; 37 -&gt; 40 -&gt; 43 -&gt; 45</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3457,6 +3597,12 @@
           <t>Shield skill. Reduce magic damage taken by the party once.</t>
         </is>
       </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Damage reduction rate: 12% -&gt; 14 -&gt; 16 -&gt; 18 -&gt; 20 -&gt; 22 -&gt; 24 -&gt; 26 -&gt; 28 -&gt; 30%
+Turns: 5   |   TP Cost: 20 -&gt; 23 -&gt; 26 -&gt; 29 -&gt; 31 -&gt; 34 -&gt; 37 -&gt; 40 -&gt; 43 -&gt; 45</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3477,6 +3623,12 @@
           <t>Short-range skill. Deal lightning damage to an enemy row. May paralyze.</t>
         </is>
       </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>ATK: 96% -&gt; 100 -&gt; 104 -&gt; 108 -&gt; 113 -&gt; 118 -&gt; 123 -&gt; 128 -&gt; 133 -&gt; 138% (L10)
+Paralysis: 20% (+2-3%/Lv) -&gt; 40%   |   TP Cost: 26 (+4-5/Lv) -&gt; 64   |   Speed: 0.8x</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3497,6 +3649,12 @@
           <t>Lance skill. Deal wind damage to one enemy. May silence.</t>
         </is>
       </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>ATK: 135% -&gt; 149 -&gt; 163 -&gt; 176 -&gt; 189 -&gt; 201 -&gt; 213 -&gt; 223 -&gt; 234 -&gt; 245% (L10)
+Silence: 20% (+3-4%/Lv) -&gt; 50%   |   Accuracy: +15%   |   TP Cost: 7 (+3/Lv) -&gt; 34</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3517,6 +3675,12 @@
           <t>Lance skill. 3-5 hits on random enemies. Stronger with a Heavy Lance.</t>
         </is>
       </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>ATK: 116% -&gt; 118 -&gt; 120 -&gt; 124 -&gt; 128 -&gt; 132 -&gt; 136 -&gt; 140 -&gt; 146 -&gt; 152% (L10)
+Heavy Lance bonus: +20%   |   TP Cost: 36 (+3-6/Lv) -&gt; 71   |   Speed: 0.7x -&gt; 0.8x</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3537,6 +3701,12 @@
           <t>Sword/lance skill. Pierces through to the back row.</t>
         </is>
       </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>ATK: 120% -&gt; 130 -&gt; 142 -&gt; 154 -&gt; 165 -&gt; 176 -&gt; 186 -&gt; 196 -&gt; 204 -&gt; 212% (L10)
+Accuracy: +5% (+1-2%/Lv) -&gt; +15%   |   TP Cost: 32 (+3/Lv) -&gt; 59   |   Speed: 0.8x</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -3557,6 +3727,12 @@
           <t>Deal increased physical damage next turn.</t>
         </is>
       </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Damage: 2.05x -&gt; 2.1x -&gt; 2.16x -&gt; 2.22x -&gt; 2.3x (L1-5 Max)
+Turns: 2   |   TP Cost: 15 -&gt; 18 -&gt; 21 -&gt; 24 -&gt; 27   |   Speed: 0.84x -&gt; 0.9x</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -3577,6 +3753,12 @@
           <t>Steal pocket money from an enemy.</t>
         </is>
       </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Steal success: 40% -&gt; 45% -&gt; 50% -&gt; 57% -&gt; 64% (L1-5 Max)
+Speed: 1x -&gt; 1.5x</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -3597,6 +3779,12 @@
           <t>Steal an item from an enemy.</t>
         </is>
       </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Steal success: 30% -&gt; 35% -&gt; 40% -&gt; 45% -&gt; 50% (L1-5 Max)
+Speed: 0.6x -&gt; 0.8x</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -3617,6 +3805,12 @@
           <t>Dagger skill. Inflict a critical hit with stab damage.</t>
         </is>
       </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>ATK: 105% -&gt; 109 -&gt; 113 -&gt; 116 -&gt; 119 -&gt; 121 -&gt; 123 -&gt; 125 -&gt; 127 -&gt; 129% (L10)
+TP Cost: 5 -&gt; 8 -&gt; 11 -&gt; 14 -&gt; 17 -&gt; 20 -&gt; 23 -&gt; 26 -&gt; 28 -&gt; 30   |   Speed: 0.9x</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -3637,6 +3831,12 @@
           <t>Dagger skill. Inflict stab damage relative to enemy's total buffs and debuffs.</t>
         </is>
       </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>ATK: 170% -&gt; 182% -&gt; 194% -&gt; 204% -&gt; 212% (L1-5 Max)
+TP Cost: 24 -&gt; 28 -&gt; 32 -&gt; 35 -&gt; 38   |   Speed: 0.85x</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -3657,6 +3857,12 @@
           <t>Increase own physical evasion rate.</t>
         </is>
       </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Evasion: +10% -&gt; +13% -&gt; +16% -&gt; +18% -&gt; +20% (L1-5 Max)
+Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8   |   TP Cost: 4 -&gt; 6 -&gt; 8 -&gt; 10 -&gt; 12</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -3677,6 +3883,12 @@
           <t>Cure status ailments for a single ally.</t>
         </is>
       </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Cures: poison &gt; paralysis &gt; silence &gt; freeze &gt; sleep
+TP Cost: 3 -&gt; 4 -&gt; 5 -&gt; 6 -&gt; 7 (L1-5 Max)</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3697,6 +3909,12 @@
           <t>Increase own accuracy.</t>
         </is>
       </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Accuracy: +15% -&gt; +17 -&gt; +19 -&gt; +21 -&gt; +23 -&gt; +25 -&gt; +26 -&gt; +27 -&gt; +28 -&gt; +30% (L10)
+Turns: 5 -&gt; 9   |   TP Cost: 5 -&gt; 8 -&gt; 11 -&gt; 14 -&gt; 17 -&gt; 20 -&gt; 22 -&gt; 24 -&gt; 26 -&gt; 28</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3717,6 +3935,12 @@
           <t>Increase own speed.</t>
         </is>
       </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Speed increase: 10% -&gt; 11 -&gt; 12 -&gt; 13 -&gt; 14 -&gt; 15 -&gt; 16 -&gt; 17 -&gt; 18 -&gt; 20% (L10)
+Turns: 3 (Lv1-3) -&gt; 4 (Lv4-6) -&gt; 5 (Lv7-9) -&gt; 6 (L10)   |   TP Cost: 14 (+2/Lv) -&gt; 32</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3737,6 +3961,12 @@
           <t>Increase own physical evasion rate and magical evasion rate.</t>
         </is>
       </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Physical evasion: +15% (+2-3%/Lv) -&gt; +25%   |   Magic evasion: +10% (+2-3%/Lv) -&gt; +20%
+Turns: 3 -&gt; 4 -&gt; 5 -&gt; 6 -&gt; 7   |   TP Cost: 12 -&gt; 14 -&gt; 16 -&gt; 18 -&gt; 20   |   Speed: 0.9x</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3757,6 +3987,12 @@
           <t>Short-range skill. Attack one enemy. May cause sleep.</t>
         </is>
       </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>ATK: 116% -&gt; 120 -&gt; 124 -&gt; 128 -&gt; 132 -&gt; 136 -&gt; 140 -&gt; 144 -&gt; 150 -&gt; 156% (L10)
+Sleep: 20% (+3-4%/Lv) -&gt; 50%   |   TP Cost: 7 (+2/Lv) -&gt; 25   |   Speed: 0.9x</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3777,6 +4013,12 @@
           <t>Short-range skill. Attack one enemy. May silence.</t>
         </is>
       </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>ATK: 116% -&gt; 120 -&gt; 124 -&gt; 128 -&gt; 132 -&gt; 136 -&gt; 140 -&gt; 144 -&gt; 150 -&gt; 156% (L10)
+Silence: 20% (+3-4%/Lv) -&gt; 50%   |   TP Cost: 7 (+2/Lv) -&gt; 25   |   Speed: 0.9x</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -3797,6 +4039,12 @@
           <t>Short-range skill. Attack one enemy. May stun.</t>
         </is>
       </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>ATK: 112% -&gt; 116 -&gt; 120 -&gt; 124 -&gt; 128 -&gt; 132 -&gt; 136 -&gt; 140 -&gt; 144 -&gt; 150% (L10)
+Stun: 20% (+3-4%/Lv) -&gt; 50%   |   TP Cost: 7 (+2/Lv) -&gt; 25   |   Speed: 0.9x</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3817,6 +4065,12 @@
           <t>Bow/gun skill. Attack one enemy multiple times with escalating crit rate.</t>
         </is>
       </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Number of attacks: 3 (Lv1-4) -&gt; 4 (Lv5-8) -&gt; 5 (L9-10)   |   ATK: 104% -&gt; 148%
+Power decrease: 25% -&gt; 14%   |   TP Cost: 30 (+4-6/Lv) -&gt; 72   |   Speed: 0.75x -&gt; 0.85x</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -3837,6 +4091,12 @@
           <t>Bow/gun skill. Fire a single shot certain to hit one enemy.</t>
         </is>
       </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>ATK: 114% -&gt; 118% -&gt; 122% -&gt; 126% -&gt; 130% (L1-5 Max)
+TP Cost: 8 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16   |   Speed: 1x -&gt; 1.12x</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3857,6 +4117,12 @@
           <t>Bow skill. Shoot a powerful single shot at one enemy for stab damage.</t>
         </is>
       </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Damage: 3.3x -&gt; 3.45x -&gt; 3.6x -&gt; 3.8x -&gt; 4x (L1-5 Max)   |   ATK: 88%
+TP Cost: 42 -&gt; 50 -&gt; 57 -&gt; 63 -&gt; 68   |   Speed: 0.4x</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3877,6 +4143,12 @@
           <t>Bow/gun skill. Attack one enemy. May poison.</t>
         </is>
       </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>ATK: 118% -&gt; 125 -&gt; 132 -&gt; 139 -&gt; 146 -&gt; 152 -&gt; 158 -&gt; 162 -&gt; 166 -&gt; 170% (L10)
+Poison: 20% (+3-4%/Lv) -&gt; 50%   |   TP Cost: 7 (+2/Lv) -&gt; 25</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3897,6 +4169,12 @@
           <t>Bow skill. Deal stab damage to one enemy. May freeze.</t>
         </is>
       </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>ATK: 118% -&gt; 125 -&gt; 132 -&gt; 139 -&gt; 146 -&gt; 152 -&gt; 158 -&gt; 162 -&gt; 166 -&gt; 170% (L10)
+Freeze: 20% (+3-4%/Lv) -&gt; 50%   |   TP Cost: 8 (+2/Lv) -&gt; 26</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3917,6 +4195,12 @@
           <t>Bow skill. Deal stab damage to one enemy. May paralyze.</t>
         </is>
       </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>ATK: 118% -&gt; 125 -&gt; 132 -&gt; 139 -&gt; 146 -&gt; 152 -&gt; 158 -&gt; 162 -&gt; 166 -&gt; 170% (L10)
+Paralysis: 20% (+3-4%/Lv) -&gt; 50%   |   TP Cost: 8 (+2/Lv) -&gt; 26</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3937,6 +4221,12 @@
           <t>Bow skill. Deal stab damage to one enemy. May slow.</t>
         </is>
       </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>ATK: 116% -&gt; 122 -&gt; 128 -&gt; 134 -&gt; 140 -&gt; 145 -&gt; 150 -&gt; 155 -&gt; 160 -&gt; 165% (L10)
+Slow: 20% (+3-4%/Lv) -&gt; 50%   |   TP Cost: 9 (+2/Lv) -&gt; 27   |   Speed: 0.95x</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3957,6 +4247,12 @@
           <t>Bow skill. Shoot a barrage of arrows that rains upon all enemies.</t>
         </is>
       </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>ATK: 84% -&gt; 88 -&gt; 92 -&gt; 96 -&gt; 100 -&gt; 103 -&gt; 106 -&gt; 109 -&gt; 112 -&gt; 115% (L10)
+TP Cost: 20 -&gt; 23 -&gt; 27 -&gt; 30 -&gt; 33 -&gt; 36 -&gt; 39 -&gt; 42 -&gt; 45 -&gt; 48   |   Speed: 0.65x</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3977,6 +4273,12 @@
           <t>Bow skill. Shower enemies with a rain of arrows across multiple turns.</t>
         </is>
       </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>ATK: 100% -&gt; 102 -&gt; 104 -&gt; 106 -&gt; 108 -&gt; 110 -&gt; 112 -&gt; 114 -&gt; 117 -&gt; 120% (L10)
+1-3 hits   |   Turns: 2 (Lv1-9) -&gt; 3 (L10 Max)   |   TP Cost: 35 (+3/Lv) -&gt; 62</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3997,6 +4299,12 @@
           <t>Bow skill. Deal stab damage to one enemy and pierce to the back row.</t>
         </is>
       </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>ATK: 130% -&gt; 144 -&gt; 158 -&gt; 171 -&gt; 184 -&gt; 196 -&gt; 207 -&gt; 217 -&gt; 226 -&gt; 234% (L10)
+Critical rate: 5% (+1-3%/Lv) -&gt; 25%   |   TP Cost: 24 (+3-4/Lv) -&gt; 55   |   Speed: 0.7x</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -4017,6 +4325,12 @@
           <t>Projectile skill. Attack and decrease speed for an enemy row.</t>
         </is>
       </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>ATK: 94% (+3-6%/Lv) -&gt; 130% | Speed decrease chance: 30% -&gt; 75% | Speed decrease: 10%
+Turns: 4   |   TP Cost: 24 -&gt; 27 -&gt; 30 -&gt; 33 -&gt; 36 -&gt; 39 -&gt; 42 -&gt; 45 -&gt; 48 -&gt; 50</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -4037,6 +4351,12 @@
           <t>Deal bash damage to one enemy. May stun.</t>
         </is>
       </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>ATK: 120% -&gt; 126 -&gt; 132 -&gt; 139 -&gt; 146 -&gt; 154 -&gt; 162 -&gt; 170 -&gt; 180 -&gt; 192% (L10)
+Stun: 10% -&gt; 20%   |   TP Cost: 12 -&gt; 15 -&gt; 18 -&gt; 21 -&gt; 24 -&gt; 27 -&gt; 30 -&gt; 32 -&gt; 34 -&gt; 36</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -4057,6 +4377,12 @@
           <t>Identify unknown items.</t>
         </is>
       </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Identification success rate: 32% -&gt; 44% -&gt; 56% -&gt; 68% -&gt; 80% (L1-5 Max)
+TP Cost: 10 -&gt; 8 -&gt; 6 -&gt; 4 -&gt; 2</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -4077,6 +4403,12 @@
           <t>Briefly sacrifice magic accuracy to increase magic damage.</t>
         </is>
       </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Magic damage: +38% -&gt; +42% -&gt; +47% -&gt; +53% -&gt; +60% (L1-5 Max)
+Magic accuracy: -2% (-2%/Lv)   |   Turns: 6   |   TP Cost: 20 -&gt; 23 -&gt; 26 -&gt; 29 -&gt; 32</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -4097,6 +4429,12 @@
           <t>Mace skill. Deal bash damage with an inexorable thud.</t>
         </is>
       </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Damage: 2x -&gt; 2.2 -&gt; 2.4 -&gt; 2.6 -&gt; 2.8 -&gt; 3 -&gt; 3.25 -&gt; 3.5 -&gt; 3.75 -&gt; 4x (L10)
+Accuracy: +10% (+2-4%/Lv) -&gt; +30%   |   ATK: 82%   |   TP Cost: 28 (+4/Lv) -&gt; 64</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -4117,6 +4455,12 @@
           <t>Mace skill. Decrease the enemy's DEF as you attack.</t>
         </is>
       </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>ATK: 135% -&gt; 147 -&gt; 159 -&gt; 171 -&gt; 183 -&gt; 193 -&gt; 203 -&gt; 213 -&gt; 220 -&gt; 225%   |   DEF: -10%
+Turns: 4   |   TP Cost: 25 -&gt; 29 -&gt; 33 -&gt; 37 -&gt; 41 -&gt; 45 -&gt; 48 -&gt; 51 -&gt; 54 -&gt; 57</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -4137,6 +4481,12 @@
           <t>Sword skill. Deal slash damage to all enemies.</t>
         </is>
       </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>ATK: 120% -&gt; 124 -&gt; 128 -&gt; 132 -&gt; 136 -&gt; 140 -&gt; 144 -&gt; 148 -&gt; 154 -&gt; 160% (L10)
+TP Cost: 36 -&gt; 40 -&gt; 44 -&gt; 48 -&gt; 52 -&gt; 57 -&gt; 62 -&gt; 67 -&gt; 73 -&gt; 79</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -4157,6 +4507,12 @@
           <t>Reduce magic damage taken for the party.</t>
         </is>
       </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Damage reduction: 18% -&gt; 20 -&gt; 22 -&gt; 24 -&gt; 26 -&gt; 28 -&gt; 30 -&gt; 32 -&gt; 34 -&gt; 36% (L10)
+Turns: 4 -&gt; 7   |   TP Cost: 22 -&gt; 25 -&gt; 28 -&gt; 31 -&gt; 34 -&gt; 38 -&gt; 42 -&gt; 46 -&gt; 50 -&gt; 56</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -4177,6 +4533,12 @@
           <t>Transform to increase own overall stats.</t>
         </is>
       </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Stat: +20% -&gt; +23% -&gt; +26% -&gt; +29% -&gt; +32% (L1-5 Max)
+Turns: 4 -&gt; 4 -&gt; 5 -&gt; 5 -&gt; 6   |   TP Cost: 52 -&gt; 60 -&gt; 70 -&gt; 80 -&gt; 92   |   Speed: 1.25x</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -4197,6 +4559,12 @@
           <t>Short-range skill. Perform a powerful lightning strike to one enemy.</t>
         </is>
       </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>ATK: 136% -&gt; 142 -&gt; 148 -&gt; 155 -&gt; 162 -&gt; 172 -&gt; 182 -&gt; 193 -&gt; 204 -&gt; 216% (L10)
+Accuracy: +10% (+1-2%/Lv) -&gt; +20%   |   TP Cost: 13 (+3-4/Lv) -&gt; 45   |   Speed: 0.9x -&gt; 1x</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -4217,6 +4585,12 @@
           <t>Tome skill. RES-based bash damage to one enemy. May freeze/silence.</t>
         </is>
       </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>ATK: 150% -&gt; 162 -&gt; 174 -&gt; 186 -&gt; 198 -&gt; 208 -&gt; 218 -&gt; 228 -&gt; 236 -&gt; 244% (L10)
+Freeze: 20% (+3-4%/Lv) -&gt; 50%   |   Silence: 20% -&gt; 50%   |   TP Cost: 9 (+3/Lv) -&gt; 36</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -4237,6 +4611,12 @@
           <t>Protect allies from gas and damage traps.</t>
         </is>
       </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Turns: 6 -&gt; 8 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16 -&gt; 18 -&gt; 20 -&gt; 22 -&gt; 24
+TP Cost: 24 -&gt; 28 -&gt; 32 -&gt; 36 -&gt; 40 -&gt; 43 -&gt; 46 -&gt; 49 -&gt; 52 -&gt; 55</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -4257,6 +4637,7 @@
           <t>Detect how many unopened treasure chests are left on the current floor.</t>
         </is>
       </c>
+      <c r="E65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -4277,6 +4658,11 @@
           <t>Heal an ally's HP.</t>
         </is>
       </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>HP recovery: 12% -&gt; 15% -&gt; 18% -&gt; 21% -&gt; 25% (L1-5 Max)</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -4297,6 +4683,12 @@
           <t>Heal an ally's TP.</t>
         </is>
       </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>TP recovery: 10% -&gt; 11% -&gt; 12% -&gt; 13% -&gt; 15% (L1-5 Max)
+Speed: 0.85x</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -4317,6 +4709,11 @@
           <t>Distribute all of one's TP to the target.</t>
         </is>
       </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>TP transfer bonus: 100% -&gt; 110% -&gt; 120% -&gt; 130% -&gt; 140% (L1-5 Max)</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -4337,6 +4734,12 @@
           <t>Clean one's surroundings in order to increase mobility.</t>
         </is>
       </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Speed increase: 12% -&gt; 14% -&gt; 16% -&gt; 18% -&gt; 20% (L1-5 Max)
+Turns: 6 -&gt; 7 -&gt; 8 -&gt; 9 -&gt; 10</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -4357,6 +4760,12 @@
           <t>Recover some TP.</t>
         </is>
       </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>TP recovery: 16% -&gt; 18% -&gt; 20% -&gt; 22% -&gt; 25% (L1-5 Max)
+Speed: 0.9x</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -4377,6 +4786,12 @@
           <t>Dance skill. Lower all enemies' ATK while dance lasts.</t>
         </is>
       </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ATK: -4% -&gt; -6 -&gt; -8 -&gt; -10 -&gt; -11 -&gt; -12 -&gt; -13 -&gt; -14 -&gt; -15 -&gt; -16% (L10)
+Speed: 0.75x</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -4397,6 +4812,12 @@
           <t>Dance skill. Lower all enemies' DEF while dance lasts.</t>
         </is>
       </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>DEF: -5% -&gt; -7 -&gt; -9 -&gt; -11 -&gt; -13 -&gt; -15 -&gt; -17 -&gt; -19 -&gt; -21 -&gt; -23% (L10)
+Speed: 0.75x</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -4417,6 +4838,12 @@
           <t>Dance skill. Lower all enemies' accuracy while dance lasts.</t>
         </is>
       </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Accuracy: -4% -&gt; -5 -&gt; -6 -&gt; -7 -&gt; -8 -&gt; -9 -&gt; -10 -&gt; -11 -&gt; -12 -&gt; -13% (L10)
+Speed: 0.75x</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -4437,6 +4864,12 @@
           <t>Dance skill. Lower all enemies' evasion while dance lasts.</t>
         </is>
       </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Evasion: -5% -&gt; -7 -&gt; -9 -&gt; -11 -&gt; -13 -&gt; -15 -&gt; -17 -&gt; -19 -&gt; -21 -&gt; -23% (L10)
+Speed: 0.75x</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -4457,6 +4890,12 @@
           <t>Dance skill. Damage all enemies at the start of user's turn while dance lasts.</t>
         </is>
       </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Max HP damage: 3% -&gt; 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 -&gt; 9 -&gt; 10 -&gt; 11 -&gt; 12% (L10)
+Total damage cap: 250 -&gt; 275 -&gt; 300 -&gt; 325 -&gt; 350 -&gt; 375 -&gt; 400 -&gt; 430 -&gt; 460 -&gt; 500</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -4477,6 +4916,12 @@
           <t>Dance skill. Lower all enemies' speed while dance lasts.</t>
         </is>
       </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Speed decrease: 5% -&gt; 6 -&gt; 7 -&gt; 8 -&gt; 9 -&gt; 10 -&gt; 11 -&gt; 12 -&gt; 13 -&gt; 14% (L10)
+Speed: 0.75x</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -4497,6 +4942,12 @@
           <t>Dance skill. Lower all enemies' elemental resistances while dance lasts.</t>
         </is>
       </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Resistance decrease: 7 -&gt; 9 -&gt; 11 -&gt; 13 -&gt; 15 -&gt; 17 -&gt; 19 -&gt; 21 -&gt; 23 -&gt; 25 (L10)
+Speed: 0.75x</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -4517,6 +4968,12 @@
           <t>Whip skill. Deal bash damage to an enemy row from mid-range.</t>
         </is>
       </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>ATK: 120% -&gt; 124 -&gt; 128 -&gt; 132 -&gt; 136 -&gt; 140 -&gt; 145 -&gt; 150 -&gt; 155 -&gt; 160% (L10)
+Power decrease: 10%   |   TP Cost: 22 (+3-4/Lv) -&gt; 50   |   Speed: 0.75x -&gt; 0.85x</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -4537,6 +4994,12 @@
           <t>Whip skill. Attack one enemy 1-5 times from mid-range.</t>
         </is>
       </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>ATK: 107% -&gt; 114% -&gt; 121% -&gt; 128% -&gt; 136% (L1-5 Max)
+TP Cost: 30 -&gt; 34 -&gt; 38 -&gt; 42 -&gt; 46   |   Speed: 0.75x -&gt; 0.8x</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -4557,6 +5020,12 @@
           <t>Whip skill. Deal bash damage to one enemy twice. May silence/paralyze.</t>
         </is>
       </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>ATK: 135% -&gt; 142% -&gt; 149% -&gt; 157% -&gt; 165% (L1-5 Max)   |   Silence: 25% (+3%/Lv)
+Paralysis: 20% -&gt; 23% -&gt; 26% -&gt; 29% -&gt; 32%   |   TP Cost: 20 -&gt; 24 -&gt; 28 -&gt; 32 -&gt; 36</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -4577,6 +5046,12 @@
           <t>Attack 0-4 times on random targets.</t>
         </is>
       </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>ATK: 104% -&gt; 108 -&gt; 112 -&gt; 116 -&gt; 120 -&gt; 124 -&gt; 127 -&gt; 130 -&gt; 133 -&gt; 136% (L10)
+Accuracy: +20%   |   TP Cost: 27 -&gt; 30 -&gt; 33 -&gt; 36 -&gt; 40 -&gt; 44 -&gt; 48 -&gt; 52 -&gt; 56 -&gt; 60</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -4597,6 +5072,12 @@
           <t>Take a break to heal own HP and raise Pep.</t>
         </is>
       </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>HP recovery: 20% -&gt; 25% -&gt; 30% -&gt; 35% -&gt; 40% (L1-5 Max)
+TP Cost: 6 -&gt; 7 -&gt; 8 -&gt; 9 -&gt; 10   |   Speed: 1.5x</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -4617,6 +5098,7 @@
           <t>Spin the magic roulette. Nobody knows what will happen.</t>
         </is>
       </c>
+      <c r="E83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -4637,6 +5119,12 @@
           <t>Attack one enemy. May instakill.</t>
         </is>
       </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>ATK: 120% -&gt; 126 -&gt; 132 -&gt; 138 -&gt; 142 -&gt; 150 -&gt; 158 -&gt; 168 -&gt; 178 -&gt; 190% (L10)
+Instakill: 15% (+1-2%/Lv) -&gt; 25%   |   TP Cost: 17 (+2/Lv) -&gt; 35   |   Speed: 0.88x</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -4657,6 +5145,12 @@
           <t>50/50 chance of non-elemental damage to each enemy. May stun.</t>
         </is>
       </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>ATK: 95% -&gt; 99 -&gt; 103 -&gt; 107 -&gt; 111 -&gt; 115 -&gt; 119 -&gt; 123 -&gt; 127 -&gt; 131% (L10)
+Stun: 40% (+3-4%/Lv) -&gt; 70%   |   TP Cost: 32 (+2/Lv) -&gt; 50   |   Speed: 0.65x</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -4677,6 +5171,12 @@
           <t>Increase own ATK at the price of lowering own DEF.</t>
         </is>
       </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>ATK: 15% (+5%/Lv) -&gt; 35% (L5 Max)   |   DEF: -11% -&gt; -14% -&gt; -17% -&gt; -21% -&gt; -25%
+Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8   |   TP Cost: 8 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -4697,6 +5197,7 @@
           <t>Open a magic box. Nobody knows what will happen.</t>
         </is>
       </c>
+      <c r="E87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -4717,6 +5218,12 @@
           <t>Turn a weakened enemy into food. Ineffective against some enemies.</t>
         </is>
       </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Conversion success: 35% -&gt; 42% -&gt; 49% -&gt; 57% -&gt; 65% (L1-5 Max)
+TP Cost: 24 -&gt; 26 -&gt; 28 -&gt; 30 -&gt; 32   |   Speed: 0.85x</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -4737,6 +5244,12 @@
           <t>Deal non-elemental damage to all enemies with a storm of roses. May poison.</t>
         </is>
       </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>ATK: 118% -&gt; 125 -&gt; 132 -&gt; 139 -&gt; 146 -&gt; 152 -&gt; 158 -&gt; 164 -&gt; 170 -&gt; 176% (L10)
+Poison: 50% (+3-4%/Lv) -&gt; 80%   |   TP Cost: 22 (+4/Lv) -&gt; 58   |   Speed: 0.6x -&gt; 0.7x</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -4757,6 +5270,12 @@
           <t>Fan skill. Deal bashing damage to one enemy. May delay enemy turn.</t>
         </is>
       </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>ATK: 150% -&gt; 162 -&gt; 174 -&gt; 186 -&gt; 198 -&gt; 208 -&gt; 218 -&gt; 228 -&gt; 240 -&gt; 256% (L10)
+Turn delay rate: 25% (+2%/Lv)   |   TP Cost: 10 (+2-3/Lv) -&gt; 32   |   Speed: 0.95x</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -4777,6 +5296,12 @@
           <t>Fan skill. With increased ATK, deal long-range damage to one enemy.</t>
         </is>
       </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>ATK: 120%
+Speed: 1.15x</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -4797,6 +5322,12 @@
           <t>Short-range skill. Pierce through to the back row with stab damage. May slow.</t>
         </is>
       </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>ATK: 130% (+8%/Lv) -&gt; 202% (L10 Max)   |   Slow: 25% -&gt; 45%   |   Accuracy: -5% (+2%/Lv)
+TP Cost: 24 -&gt; 27 -&gt; 30 -&gt; 33 -&gt; 36 -&gt; 39 -&gt; 42 -&gt; 45 -&gt; 48 -&gt; 50   |   Speed: 0.75x</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -4817,6 +5348,12 @@
           <t>Short-range skill. Attack one enemy and reduce target's max HP.</t>
         </is>
       </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>ATK: 88% -&gt; 92% -&gt; 97% -&gt; 103% -&gt; 110% (L1-5 Max)   |   Max HP reduction: 50% -&gt; 100%
+Turns: 6   |   TP Cost: 15 -&gt; 18 -&gt; 21 -&gt; 23 -&gt; 25   |   Speed: 0.85x</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -4837,6 +5374,12 @@
           <t>Convert current DEF to bonus ATK (DEF becomes 0).</t>
         </is>
       </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>DEF conversion bonus: 60% -&gt; 80% -&gt; 100% -&gt; 125% -&gt; 150% (L1-5 Max)
+Turns: 2   |   TP Cost: 38 -&gt; 41 -&gt; 44 -&gt; 47 -&gt; 50   |   Speed: 1.15x</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -4857,6 +5400,7 @@
           <t>Something emerges from the shadows. Nobody knows what will happen.</t>
         </is>
       </c>
+      <c r="E95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -4877,6 +5421,12 @@
           <t>Whip skill. Attack one enemy 1-3 times from mid-range. Crits against Beasts.</t>
         </is>
       </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>ATK: 118% -&gt; 122 -&gt; 126 -&gt; 130 -&gt; 134 -&gt; 138 -&gt; 142 -&gt; 145 -&gt; 148 -&gt; 151% (L10)
+Accuracy UP   |   TP Cost: 18 -&gt; 20 -&gt; 22 -&gt; 24 -&gt; 26 -&gt; 28 -&gt; 31 -&gt; 34 -&gt; 37 -&gt; 40</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -4897,6 +5447,12 @@
           <t>Summon Spartan for short-range bash damage.</t>
         </is>
       </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>ATK: 144% -&gt; 147 -&gt; 150 -&gt; 154 -&gt; 158 -&gt; 162 -&gt; 166 -&gt; 170 -&gt; 175 -&gt; 180% (L10)
+Turns: 3 (Lv1-3) -&gt; 4 (Lv4-6) -&gt; 5 (Lv7-9) -&gt; 6 (L10)   |   TP Cost: 20 -&gt; 42</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -4917,6 +5473,12 @@
           <t>Summon Oracles for mid-range INT-based damage and possible paralysis.</t>
         </is>
       </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>ATK: 126% (+2-5%/Lv) -&gt; 157%   |   Paralysis: 30% (+3-5%/Lv) -&gt; 64% (L10)
+Turns: 3 (Lv1-4) -&gt; 4 (Lv5-8) -&gt; 5 (Lv9-10)   |   TP Cost: 24 -&gt; 48   |   Speed: 0.9x</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -4937,6 +5499,12 @@
           <t>Summon Catalina to heal allies' HP.</t>
         </is>
       </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Heal Power: 4 -&gt; 6 -&gt; 8 -&gt; 10 -&gt; 12 (L1-5 Max)
+Turns: 3 (Lv1-2) -&gt; 4 (Lv3-4) -&gt; 5 (L5 Max)   |   TP Cost: 30 -&gt; 48   |   Speed: 0.9x</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -4957,6 +5525,12 @@
           <t>Summon Mercidarian for random long-range stab damage to all foes.</t>
         </is>
       </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>ATK: 100% -&gt; 104 -&gt; 108 -&gt; 112 -&gt; 118 -&gt; 123 -&gt; 128 -&gt; 133 -&gt; 138 -&gt; 143% (L10)
+Turns: 2 (Lv1-4) -&gt; 3 (Lv5-7) -&gt; 4 (Lv8-10)   |   TP Cost: 42 -&gt; 70   |   Speed: 0.75x</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -4977,6 +5551,12 @@
           <t>Summon Perdurabo to cure two allies' status ailments.</t>
         </is>
       </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Cures: poison &gt; paralysis &gt; silence &gt; freeze &gt; sleep &gt; petrify &gt; slow &gt; all debuffs
+Duration: 5   |   TP Cost: 22 -&gt; 24 -&gt; 26 -&gt; 28 -&gt; 30 -&gt; 32 -&gt; 34 -&gt; 38   |   Speed: 1.15x</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -4997,6 +5577,12 @@
           <t>Summon Musiy for immediate single-target attack magic.</t>
         </is>
       </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Pwr: 180 -&gt; 240 -&gt; 310 -&gt; 390 -&gt; 480 -&gt; 585 -&gt; 700 (L7 Max)
+Turns: 4   |   TP Cost: 38 (+4-6/Lv) -&gt; 68   |   Speed: 0.82x -&gt; 0.92x</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -5017,6 +5603,12 @@
           <t>Actual course of action</t>
         </is>
       </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -5037,6 +5629,12 @@
           <t>Actual course of action</t>
         </is>
       </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -5057,6 +5655,12 @@
           <t>Actual course of action</t>
         </is>
       </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -5077,6 +5681,12 @@
           <t>Actual course of action</t>
         </is>
       </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -5097,6 +5707,12 @@
           <t>Actual course of action</t>
         </is>
       </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -5117,6 +5733,12 @@
           <t>Actual course of action</t>
         </is>
       </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -5137,6 +5759,12 @@
           <t>Actual course of action</t>
         </is>
       </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -5157,6 +5785,12 @@
           <t>Poison all enemies.</t>
         </is>
       </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -5177,6 +5811,12 @@
           <t>Freeze all enemies.</t>
         </is>
       </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -5197,6 +5837,12 @@
           <t>Paralyze all enemies.</t>
         </is>
       </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -5217,6 +5863,12 @@
           <t>Silence all enemies.</t>
         </is>
       </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -5237,6 +5889,12 @@
           <t>Slow all enemies.</t>
         </is>
       </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -5257,6 +5915,12 @@
           <t>Heal one random ally for 20% of HP and TP.</t>
         </is>
       </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -5277,6 +5941,12 @@
           <t>Fully heal one enemy.</t>
         </is>
       </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -5297,6 +5967,12 @@
           <t>Deal own level x10 damage to one random ally or enemy.</t>
         </is>
       </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -5317,6 +5993,12 @@
           <t>Nothing happens.</t>
         </is>
       </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -5337,6 +6019,12 @@
           <t>Deal damage equal to own remaining HP - 1 to one random ally or enemy.</t>
         </is>
       </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -5357,6 +6045,12 @@
           <t>A long-range + stab attack to all enemies. Inflicted damage is based off the practitioner's ATK</t>
         </is>
       </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -5377,6 +6071,12 @@
           <t>Song, dance, doll, and chant are canceled for all enemies and allies.</t>
         </is>
       </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -5397,6 +6097,12 @@
           <t>Recover 75TP for the party.</t>
         </is>
       </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -5417,6 +6123,12 @@
           <t>An unknown dog (Genjimaru) appeared for support.</t>
         </is>
       </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -5437,6 +6149,12 @@
           <t>Attack oneself with own ATK.</t>
         </is>
       </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -5457,6 +6175,12 @@
           <t>Acquire the total amount of money for beating all enemies there x4.</t>
         </is>
       </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -5477,6 +6201,12 @@
           <t>Inflict a fixed damage of 666 to someone from your enemies or allies.</t>
         </is>
       </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -5497,6 +6227,12 @@
           <t>Nothing happens.</t>
         </is>
       </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -5517,6 +6253,12 @@
           <t>Instant death for the practitioner</t>
         </is>
       </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -5537,6 +6279,12 @@
           <t>Recover 200HP for the party.</t>
         </is>
       </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -5557,6 +6305,12 @@
           <t>Circle Brave and Circle Protect activated for an ally.</t>
         </is>
       </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -5577,6 +6331,12 @@
           <t>Fully recover HP for the one with the highest rate of TP loss out of your allies.</t>
         </is>
       </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -5597,6 +6357,12 @@
           <t>Stab, Cut, and Bash Protect Lv5 activated for the party.</t>
         </is>
       </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -5617,6 +6383,12 @@
           <t>Stun the party.</t>
         </is>
       </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -5637,6 +6409,12 @@
           <t>Put the party to sleep. (Guaranteed without perfect sleep resistance.)</t>
         </is>
       </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -5657,6 +6435,12 @@
           <t>Silence + freeze + slow for all enemies.</t>
         </is>
       </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -5677,6 +6461,12 @@
           <t>HP gets cut down to half for the party.</t>
         </is>
       </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -5697,6 +6487,12 @@
           <t>Aim and Fleet Foot Lv10 activated for the party.</t>
         </is>
       </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -5717,6 +6513,12 @@
           <t>HP and TP fully recovered for all enemies and allies.</t>
         </is>
       </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -5737,6 +6539,12 @@
           <t>Enemies will flee.</t>
         </is>
       </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -5757,6 +6565,12 @@
           <t>Scatter 1/10 of pocket money your ally has.</t>
         </is>
       </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -5777,6 +6591,12 @@
           <t>Attack an enemy 7 times with own ATK.</t>
         </is>
       </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -5797,6 +6617,12 @@
           <t>Nothing happens.</t>
         </is>
       </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -5817,6 +6643,12 @@
           <t>Damage one enemy for a percentage of HP.</t>
         </is>
       </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -5837,6 +6669,12 @@
           <t>Heal one enemy for a percentage of HP.</t>
         </is>
       </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -5857,6 +6695,12 @@
           <t>Deal fire damage to one enemy.</t>
         </is>
       </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>Pwr: 70 -&gt; 105 -&gt; 140 -&gt; 175 -&gt; 220 -&gt; 270 -&gt; 320 -&gt; 380 -&gt; 450 -&gt; 520 (L10)
+Accuracy: 86% (+1%/Lv)   |   TP Cost: 5 (+2-4/Lv) -&gt; 32   |   Speed: 2.25x</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -5877,6 +6721,12 @@
           <t>Deal fire damage to an enemy row.</t>
         </is>
       </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>Pwr: 90 -&gt; 120 -&gt; 160 -&gt; 200 -&gt; 240 -&gt; 290 -&gt; 340 -&gt; 400 -&gt; 460 -&gt; 530 (L10)
+Accuracy: 80% (+1-2%/Lv) -&gt; 90%   |   TP Cost: 15 (+4-6/Lv) -&gt; 60   |   Speed: 1.7x</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -5897,6 +6747,12 @@
           <t>Deal fire damage to all enemies.</t>
         </is>
       </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>Pwr: 300 -&gt; 350 -&gt; 400 -&gt; 450 -&gt; 500 -&gt; 550 -&gt; 590 -&gt; 650 -&gt; 690 -&gt; 750 (L10)
+Accuracy: 75% (+1-2%/Lv) -&gt; 85%   |   TP Cost: 42 (+6-10/Lv) -&gt; 120   |   Speed: 1.3x</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -5917,6 +6773,12 @@
           <t>Deal tremendous fire damage to one enemy.</t>
         </is>
       </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>Pwr: 620 -&gt; 760 -&gt; 920 -&gt; 1100 -&gt; 1300 (L1-5 Max)   |   Accuracy: 82% (+2%/Lv)
+TP Cost: 40 -&gt; 50 -&gt; 60 -&gt; 72 -&gt; 84   |   Speed: 1.5x   |   Chant: 0.75x -&gt; 0.7x</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -5937,6 +6799,12 @@
           <t>Deal water damage to one enemy.</t>
         </is>
       </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Pwr: 70 -&gt; 105 -&gt; 140 -&gt; 175 -&gt; 220 -&gt; 270 -&gt; 320 -&gt; 380 -&gt; 450 -&gt; 520 (L10)
+Accuracy: 86% (+1%/Lv)   |   TP Cost: 5 (+2-4/Lv) -&gt; 32   |   Speed: 2.25x</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -5957,6 +6825,12 @@
           <t>Deal water damage to an enemy row.</t>
         </is>
       </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>Pwr: 90 -&gt; 120 -&gt; 160 -&gt; 200 -&gt; 240 -&gt; 290 -&gt; 340 -&gt; 400 -&gt; 460 -&gt; 530 (L10)
+Accuracy: 80% (+1-2%/Lv) -&gt; 90%   |   TP Cost: 15 (+4-6/Lv) -&gt; 60   |   Speed: 1.7x</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -5977,6 +6851,12 @@
           <t>Deal water damage to all enemies.</t>
         </is>
       </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>Pwr: 300 -&gt; 350 -&gt; 400 -&gt; 450 -&gt; 500 -&gt; 550 -&gt; 590 -&gt; 650 -&gt; 690 -&gt; 750 (L10)
+Accuracy: 75% (+1-2%/Lv) -&gt; 85%   |   TP Cost: 42 (+6-10/Lv) -&gt; 120   |   Speed: 1.3x</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -5997,6 +6877,12 @@
           <t>Deal tremendous water damage to one enemy.</t>
         </is>
       </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>Pwr: 620 -&gt; 760 -&gt; 920 -&gt; 1100 -&gt; 1300 (L1-5 Max)   |   Accuracy: 82% (+2%/Lv)
+TP Cost: 40 -&gt; 50 -&gt; 60 -&gt; 72 -&gt; 84   |   Speed: 1.5x   |   Chant: 0.75x -&gt; 0.7x</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -6017,6 +6903,12 @@
           <t>Deal lightning damage to one enemy.</t>
         </is>
       </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>Pwr: 70 -&gt; 105 -&gt; 140 -&gt; 175 -&gt; 220 -&gt; 270 -&gt; 320 -&gt; 380 -&gt; 450 -&gt; 520 (L10)
+Accuracy: 86% (+1%/Lv)   |   TP Cost: 5 (+2-4/Lv) -&gt; 32   |   Speed: 2.25x</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -6037,6 +6929,12 @@
           <t>Deal lightning damage to an enemy row.</t>
         </is>
       </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>Pwr: 90 -&gt; 120 -&gt; 160 -&gt; 200 -&gt; 240 -&gt; 290 -&gt; 340 -&gt; 400 -&gt; 460 -&gt; 530 (L10)
+Accuracy: 80% (+1-2%/Lv) -&gt; 90%   |   TP Cost: 15 (+4-6/Lv) -&gt; 60   |   Speed: 1.7x</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -6057,6 +6955,12 @@
           <t>Deal lightning damage to all enemies.</t>
         </is>
       </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>Pwr: 300 -&gt; 350 -&gt; 400 -&gt; 450 -&gt; 500 -&gt; 550 -&gt; 590 -&gt; 650 -&gt; 690 -&gt; 750 (L10)
+Accuracy: 75% (+1-2%/Lv) -&gt; 85%   |   TP Cost: 42 (+6-10/Lv) -&gt; 120   |   Speed: 1.3x</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -6077,6 +6981,12 @@
           <t>Deal tremendous lightning damage to one enemy.</t>
         </is>
       </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>Pwr: 620 -&gt; 760 -&gt; 920 -&gt; 1100 -&gt; 1300 (L1-5 Max)   |   Accuracy: 82% (+2%/Lv)
+TP Cost: 40 -&gt; 50 -&gt; 60 -&gt; 72 -&gt; 84   |   Speed: 1.5x   |   Chant: 0.75x -&gt; 0.7x</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -6097,6 +7007,12 @@
           <t>Deal wind damage to one enemy.</t>
         </is>
       </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Pwr: 70 -&gt; 105 -&gt; 140 -&gt; 175 -&gt; 220 -&gt; 270 -&gt; 320 -&gt; 380 -&gt; 450 -&gt; 520 (L10)
+Accuracy: 86% (+1%/Lv)   |   TP Cost: 5 (+2-4/Lv) -&gt; 32   |   Speed: 2.25x</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -6117,6 +7033,12 @@
           <t>Deal wind damage to an enemy row.</t>
         </is>
       </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>Pwr: 90 -&gt; 120 -&gt; 160 -&gt; 200 -&gt; 240 -&gt; 290 -&gt; 340 -&gt; 400 -&gt; 460 -&gt; 530 (L10)
+Accuracy: 80% (+1-2%/Lv) -&gt; 90%   |   TP Cost: 15 (+4-6/Lv) -&gt; 60   |   Speed: 1.7x</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -6137,6 +7059,12 @@
           <t>Deal wind damage to all enemies.</t>
         </is>
       </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>Pwr: 300 -&gt; 350 -&gt; 400 -&gt; 450 -&gt; 500 -&gt; 550 -&gt; 590 -&gt; 650 -&gt; 690 -&gt; 750 (L10)
+Accuracy: 75% (+1-2%/Lv) -&gt; 85%   |   TP Cost: 42 (+6-10/Lv) -&gt; 120   |   Speed: 1.3x</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -6157,6 +7085,12 @@
           <t>Deal tremendous wind damage to one enemy.</t>
         </is>
       </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>Pwr: 620 -&gt; 760 -&gt; 920 -&gt; 1100 -&gt; 1300 (L1-5 Max)   |   Accuracy: 82% (+2%/Lv)
+TP Cost: 40 -&gt; 50 -&gt; 60 -&gt; 72 -&gt; 84   |   Speed: 1.5x   |   Chant: 0.75x -&gt; 0.7x</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -6177,6 +7111,12 @@
           <t>Deal earth damage to one enemy.</t>
         </is>
       </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>Pwr: 70 -&gt; 105 -&gt; 140 -&gt; 175 -&gt; 220 -&gt; 270 -&gt; 320 -&gt; 380 -&gt; 450 -&gt; 520 (L10)
+Accuracy: 86% (+1%/Lv)   |   TP Cost: 5 (+2-4/Lv) -&gt; 32   |   Speed: 2.25x</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -6197,6 +7137,12 @@
           <t>Deal earth damage to an enemy row.</t>
         </is>
       </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>Pwr: 90 -&gt; 120 -&gt; 160 -&gt; 200 -&gt; 240 -&gt; 290 -&gt; 340 -&gt; 400 -&gt; 460 -&gt; 530 (L10)
+Accuracy: 80% (+1-2%/Lv) -&gt; 90%   |   TP Cost: 15 (+4-6/Lv) -&gt; 60   |   Speed: 1.7x</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -6217,6 +7163,12 @@
           <t>Deal earth damage to all enemies.</t>
         </is>
       </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>Pwr: 300 -&gt; 350 -&gt; 400 -&gt; 450 -&gt; 500 -&gt; 550 -&gt; 590 -&gt; 650 -&gt; 690 -&gt; 750 (L10)
+Accuracy: 75% (+1-2%/Lv) -&gt; 85%   |   TP Cost: 42 (+6-10/Lv) -&gt; 120   |   Speed: 1.3x</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -6237,6 +7189,12 @@
           <t>Deal tremendous earth damage to one enemy.</t>
         </is>
       </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>Pwr: 620 -&gt; 760 -&gt; 920 -&gt; 1100 -&gt; 1300 (L1-5 Max)   |   Accuracy: 82% (+2%/Lv)
+TP Cost: 40 -&gt; 50 -&gt; 60 -&gt; 72 -&gt; 84   |   Speed: 1.5x   |   Chant: 0.75x -&gt; 0.7x</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -6257,6 +7215,12 @@
           <t>Deal non-elemental damage to one enemy to regain HP.</t>
         </is>
       </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>Pwr: 60 -&gt; 95 -&gt; 130 -&gt; 165 -&gt; 200 -&gt; 230 -&gt; 260 -&gt; 290 -&gt; 320 -&gt; 350 (L10)
+Accuracy: 80% (+1-2%/Lv) -&gt; 90%   |   HP Absorb: 100%   |   TP Cost: 9 (+1/Lv) -&gt; 18</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -6277,6 +7241,12 @@
           <t>Deal non-elemental damage to one enemy to regain TP.</t>
         </is>
       </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>Pwr: 22 -&gt; 30 -&gt; 38 -&gt; 46 -&gt; 54 -&gt; 60 -&gt; 66 -&gt; 72 -&gt; 78 -&gt; 82   |   Accuracy: 80% -&gt; 90%
+TP Absorb: 100% | TP Cost: 6 (+1/Lv) -&gt; 15 | Speed: 1.75x | Chant: 1.25x -&gt; 1.07x</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -6297,6 +7267,12 @@
           <t>Raise max HP.</t>
         </is>
       </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>Max HP increase rate: 20% -&gt; 28% -&gt; 36% -&gt; 45% -&gt; 50% (L1-5 Max)
+Turns: 6 -&gt; 7 -&gt; 8 -&gt; 9 -&gt; 10   |   TP Cost: 27 -&gt; 31 -&gt; 35 -&gt; 39 -&gt; 43   |   Speed: 1.5x</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -6317,6 +7293,12 @@
           <t>Absorb HP from an enemy row.</t>
         </is>
       </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>Pwr: 75 (+35-45/Lv) -&gt; 450   |   Accuracy: 65% (+2-3%/Lv) -&gt; 87%   |   HP Absorb: 100%
+TP Cost: 18 -&gt; 21 -&gt; 24 -&gt; 27 -&gt; 30 -&gt; 34 -&gt; 38 -&gt; 42 -&gt; 46 -&gt; 50   |   Speed: 1.5x</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -6337,6 +7319,12 @@
           <t>Stun one enemy.</t>
         </is>
       </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>Accuracy: 65% -&gt; 68% -&gt; 71% -&gt; 73% -&gt; 75% (L1-5 Max)
+TP Cost: 10 -&gt; 12 -&gt; 14 -&gt; 16 -&gt; 18   |   Speed: 0.8x -&gt; 0.92x   |   Chant: 1.25x</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -6357,6 +7345,12 @@
           <t>Poison all enemies.</t>
         </is>
       </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>Accuracy: 75% -&gt; 78% -&gt; 81% -&gt; 83% -&gt; 85% (L1-5 Max)
+TP Cost: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8   |   Speed: 2.15x   |   Chant: 1.2x -&gt; 1.4x</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -6377,6 +7371,12 @@
           <t>Freeze all enemies.</t>
         </is>
       </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>Accuracy: 70% -&gt; 72% -&gt; 74% -&gt; 76% -&gt; 78% (L1-5 Max)
+TP Cost: 6 -&gt; 7 -&gt; 8 -&gt; 9 -&gt; 10   |   Speed: 1.5x   |   Chant: 1.5x -&gt; 1.66x</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -6397,6 +7397,12 @@
           <t>Paralyze all enemies.</t>
         </is>
       </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>Accuracy: 65% -&gt; 68% -&gt; 71% -&gt; 73% -&gt; 75% (L1-5 Max)
+TP Cost: 6 -&gt; 7 -&gt; 8 -&gt; 9 -&gt; 10   |   Speed: 1.5x   |   Chant: 1x -&gt; 1.2x</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -6417,6 +7423,12 @@
           <t>Put an enemy row to sleep.</t>
         </is>
       </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>Accuracy: 65% -&gt; 68% -&gt; 71% -&gt; 73% -&gt; 75% (L1-5 Max)
+TP Cost: 10 -&gt; 12 -&gt; 14 -&gt; 16 -&gt; 18   |   Chant: 0.75x -&gt; 0.87x</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -6437,6 +7449,12 @@
           <t>Silence all enemies.</t>
         </is>
       </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>Accuracy: 70% -&gt; 72% -&gt; 74% -&gt; 76% -&gt; 78% (L1-5 Max)
+TP Cost: 6 -&gt; 7 -&gt; 8 -&gt; 9 -&gt; 10   |   Speed: 1.5x   |   Chant: 1.5x -&gt; 1.66x</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -6457,6 +7475,12 @@
           <t>Petrify an enemy row.</t>
         </is>
       </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>Accuracy: 70% -&gt; 72% -&gt; 74% -&gt; 76% -&gt; 78% (L1-5 Max)
+TP Cost: 15 -&gt; 17 -&gt; 19 -&gt; 21 -&gt; 23   |   Chant: 0.75x -&gt; 0.87x</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -6477,6 +7501,12 @@
           <t>Instakill one enemy.</t>
         </is>
       </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>Accuracy: 50% -&gt; 52% -&gt; 55% -&gt; 58% -&gt; 60% (L1-5 Max)
+TP Cost: 12 -&gt; 14 -&gt; 16 -&gt; 18 -&gt; 20   |   Chant: 0.75x -&gt; 0.87x</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -6497,6 +7527,12 @@
           <t>Slow an enemy row.</t>
         </is>
       </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>Accuracy: 50% -&gt; 55% -&gt; 60% -&gt; 64% -&gt; 68% (L1-5 Max)
+TP Cost: 15 -&gt; 17 -&gt; 19 -&gt; 21 -&gt; 23   |   Chant: 1x -&gt; 1.12x</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -6517,6 +7553,12 @@
           <t>Stun an enemy row.</t>
         </is>
       </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>Accuracy: 54% -&gt; 58% -&gt; 62% -&gt; 66% -&gt; 70% (L1-5 Max)
+TP Cost: 22 -&gt; 24 -&gt; 26 -&gt; 28 -&gt; 30   |   Speed: 0.4x -&gt; 0.5x   |   Chant: 1.25x</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -6537,6 +7579,12 @@
           <t>Negate buffs for all enemies.</t>
         </is>
       </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>Accuracy: 55% -&gt; 65% -&gt; 75% -&gt; 85% -&gt; 95% (L1-5 Max)   |   Buff cancel rate: 100%
+TP Cost: 8 -&gt; 11 -&gt; 14 -&gt; 18 -&gt; 22   |   Speed: 1.25x   |   Chant: 1.25x -&gt; 1.45x</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -6557,6 +7605,12 @@
           <t>Deal non-elemental damage to all enemies (effective vs. unholy monsters).</t>
         </is>
       </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>Pwr: 250 (+40-50/Lv) -&gt; 640   |   Accuracy: 60% -&gt; 70%   |   Damage vs. unholy: +100%
+TP Cost: 45 -&gt; 52 -&gt; 59 -&gt; 66 -&gt; 74 -&gt; 80 -&gt; 86 -&gt; 90 -&gt; 95 -&gt; 100   |   Speed: 1.75x</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -6577,6 +7631,12 @@
           <t>Imbue an ally's weapon with fire.</t>
         </is>
       </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>Turns: 6 -&gt; 7 -&gt; 8 -&gt; 9 -&gt; 10 (L1-5 Max)   |   TP Cost: 6 -&gt; 7 -&gt; 8 -&gt; 9 -&gt; 10
+Speed: 1.5x -&gt; 1.7x   |   Chant: 1.75x -&gt; 2.25x</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -6597,6 +7657,12 @@
           <t>Imbue an ally's weapon with water.</t>
         </is>
       </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>Turns: 6 -&gt; 7 -&gt; 8 -&gt; 9 -&gt; 10 (L1-5 Max)   |   TP Cost: 6 -&gt; 7 -&gt; 8 -&gt; 9 -&gt; 10
+Speed: 1.5x -&gt; 1.7x   |   Chant: 1.75x -&gt; 2.25x</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -6617,6 +7683,12 @@
           <t>Imbue an ally's weapon with lightning.</t>
         </is>
       </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>Turns: 6 -&gt; 7 -&gt; 8 -&gt; 9 -&gt; 10 (L1-5 Max)   |   TP Cost: 6 -&gt; 7 -&gt; 8 -&gt; 9 -&gt; 10
+Speed: 1.5x -&gt; 1.7x   |   Chant: 1.75x -&gt; 2.25x</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -6637,6 +7709,12 @@
           <t>Imbue an ally's weapon with wind.</t>
         </is>
       </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>Turns: 6 -&gt; 7 -&gt; 8 -&gt; 9 -&gt; 10 (L1-5 Max)   |   TP Cost: 6 -&gt; 7 -&gt; 8 -&gt; 9 -&gt; 10
+Speed: 1.5x -&gt; 1.7x   |   Chant: 1.75x -&gt; 2.25x</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -6657,6 +7735,12 @@
           <t>Imbue an ally's weapon with earth.</t>
         </is>
       </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>Turns: 6 -&gt; 7 -&gt; 8 -&gt; 9 -&gt; 10 (L1-5 Max)   |   TP Cost: 6 -&gt; 7 -&gt; 8 -&gt; 9 -&gt; 10
+Speed: 1.5x -&gt; 1.7x   |   Chant: 1.75x -&gt; 2.25x</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -6677,6 +7761,12 @@
           <t>Raise one row of allies' resistance to stab damage.</t>
         </is>
       </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>Resistance: 20 -&gt; 24 -&gt; 28 -&gt; 32 -&gt; 36 (L1-5 Max)
+Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8   |   TP Cost: 15 -&gt; 17 -&gt; 19 -&gt; 21 -&gt; 23</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -6697,6 +7787,12 @@
           <t>Raise one row of allies' resistance to slash damage.</t>
         </is>
       </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>Resistance: 18 -&gt; 24 -&gt; 28 -&gt; 32 -&gt; 36 (L1-5 Max)
+Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8   |   TP Cost: 15 -&gt; 17 -&gt; 19 -&gt; 21 -&gt; 23</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -6717,6 +7813,12 @@
           <t>Raise one row of allies' resistance to bash damage.</t>
         </is>
       </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>Resistance: 18 -&gt; 24 -&gt; 28 -&gt; 32 -&gt; 36 (L1-5 Max)
+Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8   |   TP Cost: 15 -&gt; 17 -&gt; 19 -&gt; 21 -&gt; 23</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -6737,6 +7839,12 @@
           <t>Heal an ally's HP.</t>
         </is>
       </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>Heals RES: 4x (+1x/Lv) -&gt; 13x (L10 Max)   |   Heal Cap: 100 (+60-80/Lv) -&gt; 800
+TP Cost: 3 -&gt; 5 -&gt; 7 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 17 -&gt; 20 -&gt; 23 -&gt; 26   |   Speed: 1.75x</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -6757,6 +7865,12 @@
           <t>Heal the party's HP.</t>
         </is>
       </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>Heals RES: 2.5x (+0.5x/Lv) -&gt; 7x (L10 Max)   |   Heal Cap: 80 (+50-60/Lv) -&gt; 600
+TP Cost: 15 -&gt; 20 -&gt; 25 -&gt; 30 -&gt; 35 -&gt; 40 -&gt; 46 -&gt; 52 -&gt; 58 -&gt; 64   |   Speed: 1.35x</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -6777,6 +7891,11 @@
           <t>Fully heal one ally's HP.</t>
         </is>
       </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>TP Cost: 48 -&gt; 45 -&gt; 42 -&gt; 39 -&gt; 36 (L1-5 Max)   |   Speed: 1.15x   |   Chant: 1.5x -&gt; 1.75x</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -6797,6 +7916,12 @@
           <t>Cure status ailments for a single ally.</t>
         </is>
       </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>Cures: poison &gt; paralysis &gt; silence &gt; freeze &gt; sleep &gt; petrify &gt; slow &gt; all debuffs
+TP Cost: 2 -&gt; 3 -&gt; 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 -&gt; 9   |   Speed: 2.25x   |   Chant: 2.75x</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -6817,6 +7942,12 @@
           <t>Cure party's status ailments.</t>
         </is>
       </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>Cures: poison &gt; paralysis &gt; silence &gt; freeze &gt; sleep &gt; petrify &gt; slow &gt; all debuffs
+TP Cost: 9 -&gt; 12 -&gt; 15 -&gt; 18 -&gt; 21 -&gt; 25 -&gt; 30 -&gt; 36   |   Speed: 1.5x   |   Chant: 2x</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -6837,6 +7968,12 @@
           <t>Revive a dead ally.</t>
         </is>
       </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>HP on revival: 40% -&gt; 52% -&gt; 64% -&gt; 76% -&gt; 88% (L1-5 Max)
+TP Cost: 26 -&gt; 30 -&gt; 34 -&gt; 38 -&gt; 42   |   Speed: 1.25x   |   Chant: 1.3x -&gt; 1.5x</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -6857,6 +7994,12 @@
           <t>Raise an ally's ATK.</t>
         </is>
       </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>ATK: +10% -&gt; +13% -&gt; +16% -&gt; +19% -&gt; +22% (L1-5 Max)
+Turns: 5 -&gt; 6 -&gt; 7 -&gt; 8 -&gt; 9   |   TP Cost: 9 -&gt; 11 -&gt; 13 -&gt; 15 -&gt; 17   |   Chant: 1.25x</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -6877,6 +8020,12 @@
           <t>Raise an ally's DEF.</t>
         </is>
       </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>DEF: +10% -&gt; +14% -&gt; +18% -&gt; +22% -&gt; +25% (L1-5 Max)
+Turns: 5 -&gt; 6 -&gt; 7 -&gt; 8 -&gt; 9   |   TP Cost: 9 -&gt; 11 -&gt; 13 -&gt; 15 -&gt; 17   |   Chant: 1.25x</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -6897,6 +8046,12 @@
           <t>Raise the party's magic defense.</t>
         </is>
       </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>Magic defense: +10% -&gt; +12% -&gt; +14% -&gt; +16% -&gt; +18% (L1-5 Max)
+Turns: 6 -&gt; 7 -&gt; 8 -&gt; 9 -&gt; 10   |   TP Cost: 16 -&gt; 20 -&gt; 24 -&gt; 28 -&gt; 32   |   Chant: 1.25x</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -6917,6 +8072,12 @@
           <t>Raise the party's resistance to fire, water, lightning, wind, and earth.</t>
         </is>
       </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>Elemental resistance increase: 5 -&gt; 10 -&gt; 15 -&gt; 20 -&gt; 25 (L1-5 Max)
+Turns: 6 -&gt; 7 -&gt; 8 -&gt; 9 -&gt; 10   |   TP Cost: 16 -&gt; 20 -&gt; 24 -&gt; 28 -&gt; 32   |   Chant: 1.25x</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -6937,6 +8098,12 @@
           <t>Raise an ally's speed.</t>
         </is>
       </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>Speed increase: 8% -&gt; 9% -&gt; 10% -&gt; 11% -&gt; 12% (L1-5 Max)
+Turns: 3   |   TP Cost: 15 -&gt; 18 -&gt; 21 -&gt; 24 -&gt; 27   |   Speed: 1.25x -&gt; 1.41x</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -6957,6 +8124,12 @@
           <t>Raise an ally's max HP.</t>
         </is>
       </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>Max HP: +20% -&gt; +23 -&gt; +26 -&gt; +29 -&gt; +32 -&gt; +35 -&gt; +38 -&gt; +41 -&gt; +44 -&gt; +47% (L10)
+Turns: 5 -&gt; 5 -&gt; 6 -&gt; 6 -&gt; 7 -&gt; 7 -&gt; 8 -&gt; 8 -&gt; 9 -&gt; 10   |   TP Cost: 18 (+3/Lv) -&gt; 45</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -6977,6 +8150,12 @@
           <t>Cure one row of allies' status ailments.</t>
         </is>
       </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>Cures: poison &gt; paralysis &gt; silence &gt; freeze &gt; sleep &gt; petrify &gt; slow &gt; all debuffs
+TP Cost: 7 -&gt; 10 -&gt; 13 -&gt; 16 -&gt; 19 -&gt; 21 -&gt; 24 -&gt; 28   |   Speed: 1.75x   |   Chant: 2.25x</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -6997,6 +8176,12 @@
           <t>Create 2 magical afterimages that let you dodge one attack each.</t>
         </is>
       </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>Turns: 3 -&gt; 4 -&gt; 5 (L1-3 Max)   |   TP Cost: 30 -&gt; 38 -&gt; 46   |   Speed: 0.85x
+Chant: 0.75x -&gt; 0.65x</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -7017,6 +8202,12 @@
           <t>Reduce incoming physical damage by a certain amount.</t>
         </is>
       </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>Amount of damage reduced: 30% -&gt; 33% -&gt; 37% -&gt; 41% -&gt; 45% (L1-5 Max)
+Turns: 4   |   TP Cost: 24 -&gt; 28 -&gt; 33 -&gt; 37 -&gt; 42   |   Speed: 1.5x   |   Chant: 0.75x</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -7037,6 +8228,12 @@
           <t>While active, immediately revive upon death.</t>
         </is>
       </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>Amount of HP on revival: 10% -&gt; 20% -&gt; 30% -&gt; 40% -&gt; 50% (L1-5 Max)
+Turns: 6 -&gt; 7 -&gt; 8 -&gt; 9 -&gt; 10   |   TP Cost: 25 -&gt; 30 -&gt; 35 -&gt; 40 -&gt; 45   |   Speed: 1.5x</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -7057,6 +8254,11 @@
           <t>Illuminate the dungeon to find hidden pathways.</t>
         </is>
       </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>Turns: 12 -&gt; 14 -&gt; 16 -&gt; 18 -&gt; 20 -&gt; 22 -&gt; 24 -&gt; 26 -&gt; 28 -&gt; 30</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -7077,6 +8279,11 @@
           <t>Escape from the dungeon.</t>
         </is>
       </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>TP Cost: 28 -&gt; 21 -&gt; 14 -&gt; 7 -&gt; 1 (L1-5 Max)</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -7097,6 +8304,12 @@
           <t>Put an enemy to sleep.</t>
         </is>
       </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>Accuracy: 70% -&gt; 73% -&gt; 76% -&gt; 79% -&gt; 82% (L1-5 Max)
+Speed: 1.5x   |   Chant: 1.5x -&gt; 1.66x</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -7117,6 +8330,11 @@
           <t>Raise the party's chance of doing multiple strikes while song lasts.</t>
         </is>
       </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>Speed: 1.35x   |   Chant: 1.4x</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -7137,6 +8355,12 @@
           <t>Raise the party's critical rate while song lasts.</t>
         </is>
       </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>Critical rate: 10% -&gt; 12 -&gt; 14 -&gt; 16 -&gt; 18 -&gt; 20 -&gt; 22 -&gt; 24 -&gt; 26 -&gt; 28% (L10)
+Speed: 1.35x   |   Chant: 1.4x -&gt; 2x</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -7157,6 +8381,12 @@
           <t>Raise the party's magic attack power while song lasts.</t>
         </is>
       </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>Magic attack: +10% -&gt; +11 -&gt; +12 -&gt; +13 -&gt; +14 -&gt; +15 -&gt; +16 -&gt; +17 -&gt; +18 -&gt; +20%
+Speed: 1.35x   |   Chant: 1.25x -&gt; 1.7x</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -7177,6 +8407,12 @@
           <t>Raise the party's magic defense power while song lasts.</t>
         </is>
       </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>Magic defense: +10% -&gt; +11 -&gt; +12 -&gt; +13 -&gt; +14 -&gt; +15 -&gt; +16 -&gt; +17 -&gt; +18 -&gt; +20%
+Speed: 1.35x   |   Chant: 1.25x -&gt; 1.7x</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -7197,6 +8433,12 @@
           <t>Decrease the party's chant time while song lasts.</t>
         </is>
       </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>Chant time: -10% -&gt; -11 -&gt; -12 -&gt; -13 -&gt; -14 -&gt; -15 -&gt; -16 -&gt; -17 -&gt; -18 -&gt; -20%
+Speed: 1.35x   |   Chant: 1.4x -&gt; 2x</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -7217,6 +8459,12 @@
           <t>Gradually heal the party's HP while song lasts.</t>
         </is>
       </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>HP recovery: 20 -&gt; 35 -&gt; 50 -&gt; 65 -&gt; 80 -&gt; 100 -&gt; 130 -&gt; 170 -&gt; 210 -&gt; 250 (L10)
+Speed: 1.35x   |   Chant: 1.25x -&gt; 1.7x</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -7237,6 +8485,12 @@
           <t>Gradually heal the party's TP while song lasts.</t>
         </is>
       </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>TP recovery: 4 -&gt; 6 -&gt; 8 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 18 -&gt; 22 -&gt; 26 -&gt; 30 (L10)
+Speed: 1.35x   |   Chant: 1.1x -&gt; 1.5x</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -7257,6 +8511,12 @@
           <t>Raise the party's speed while song lasts.</t>
         </is>
       </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>Speed increase: 6% -&gt; 7 -&gt; 8 -&gt; 9 -&gt; 10 -&gt; 11 -&gt; 12 -&gt; 13 -&gt; 14 -&gt; 15% (L10)
+Speed: 1.35x   |   Chant: 1.1x -&gt; 1.5x</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -7277,6 +8537,12 @@
           <t>Raise the party's acquired EXP while song lasts.</t>
         </is>
       </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>EXP: +16% -&gt; +17 -&gt; +18 -&gt; +19 -&gt; +20 -&gt; +21 -&gt; +22 -&gt; +23 -&gt; +24 -&gt; +25% (L10)
+Speed: 1.35x   |   Chant: 1.25x -&gt; 1.7x</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -7297,6 +8563,12 @@
           <t>Raise the party's magic accuracy while song lasts.</t>
         </is>
       </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>Magic accuracy: +6% -&gt; +7 -&gt; +8 -&gt; +9 -&gt; +10 -&gt; +11 -&gt; +12 -&gt; +13 -&gt; +14 -&gt; +15%
+Speed: 1.35x   |   Chant: 1.25x -&gt; 1.7x</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -7317,6 +8589,12 @@
           <t>Dodge enemy attacks by creating a shadow clone.</t>
         </is>
       </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>Number of dodges: 1 -&gt; 2 -&gt; 3 -&gt; 4 -&gt; 5 (L1-5 Max)
+Turns: 3 -&gt; 3 -&gt; 4 -&gt; 4 -&gt; 5   |   TP Cost: 23 -&gt; 27 -&gt; 32 -&gt; 38 -&gt; 45   |   Speed: 0.85x</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -7337,6 +8615,12 @@
           <t>Disable skill usage for an enemy row. Level must exceed the target's.</t>
         </is>
       </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>Shadow Sew Success: 30% -&gt; 32% -&gt; 35% -&gt; 37% -&gt; 40% (L1-5 Max)
+Turns: 3 | TP Cost: 36 -&gt; 39 -&gt; 43 -&gt; 47 -&gt; 52 | Speed: 0.8x | Chant: 0.8x -&gt; 0.88x</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -7357,6 +8641,12 @@
           <t>Lower all enemies' accuracy.</t>
         </is>
       </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>Accuracy: -10% -&gt; -12% -&gt; -14% -&gt; -16% -&gt; -18% (L1-5 Max)
+Turns: 3   |   TP Cost: 15 -&gt; 18 -&gt; 21 -&gt; 24 -&gt; 27   |   Chant: 1.15x -&gt; 1.3x</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -7377,6 +8667,12 @@
           <t>Deal fire damage based on enemy's max HP and lower ATK to an enemy row.</t>
         </is>
       </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>Max HP damage: 4% -&gt; 5% -&gt; 6% -&gt; 7% -&gt; 8% (L1-5 Max)   |   Accuracy: 64% (+4%/Lv)
+ATK: -4% (-1%/Lv) (3 Turns)   |   Damage cap: 250 -&gt; 500   |   TP Cost: 20 (+5/Lv) -&gt; 40</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -7397,6 +8693,12 @@
           <t>Deal water damage based on enemy's max HP and lower magic def. to an enemy row.</t>
         </is>
       </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>Max HP damage: 4% -&gt; 5% -&gt; 6% -&gt; 7% -&gt; 8% (L1-5 Max)   |   Accuracy: 64% (+4%/Lv)
+Magic defense: -7% -&gt; -18%   |   Damage cap: 250 -&gt; 500   |   TP Cost: 20 (+5/Lv) -&gt; 40</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -7417,6 +8719,12 @@
           <t>Deal lightning damage based on enemy's max HP and lower speed to an enemy row.</t>
         </is>
       </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>Max HP damage: 4% -&gt; 5% -&gt; 6% -&gt; 7% -&gt; 8% (L1-5 Max)   |   Accuracy: 64% (+4%/Lv)
+Speed decrease: 4% (+1%/Lv)   |   Damage cap: 250 -&gt; 500   |   TP Cost: 20 (+5/Lv) -&gt; 40</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -7437,6 +8745,12 @@
           <t>Deal wind damage based on enemy's max HP and lower evasion to an enemy row.</t>
         </is>
       </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>Max HP damage: 4% -&gt; 5% -&gt; 6% -&gt; 7% -&gt; 8% (L1-5 Max)   |   Accuracy: 64% (+4%/Lv)
+Evasion: -7% (-2%/Lv) (3 Turns)   |   Damage cap: 250 -&gt; 500   |   TP Cost: 20 (+5/Lv) -&gt; 40</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -7457,6 +8771,12 @@
           <t>Deal earth damage based on enemy's max HP and lower DEF to an enemy row.</t>
         </is>
       </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>Max HP damage: 4% -&gt; 5% -&gt; 6% -&gt; 7% -&gt; 8% (L1-5 Max)   |   Accuracy: 64% (+4%/Lv)
+DEF: -4% (-1%/Lv) (3 Turns)   |   Damage cap: 250 -&gt; 500   |   TP Cost: 20 (+5/Lv) -&gt; 40</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -7477,6 +8797,12 @@
           <t>Deal non-elemental damage to an enemy row.</t>
         </is>
       </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>Pwr: 350 -&gt; 390 -&gt; 430 -&gt; 470 -&gt; 510 -&gt; 550 -&gt; 590 -&gt; 630 -&gt; 680 -&gt; 720 (L10)
+Accuracy: 86% (+1%/Lv)   |   TP Cost: 22 (+4-6/Lv) -&gt; 66   |   Speed: 1.3x</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -7497,6 +8823,12 @@
           <t>Deal non-elemental damage to all enemies. May stun.</t>
         </is>
       </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>Pwr: 240 (+40/Lv) -&gt; 600 (L10 Max)   |   Accuracy: 76% (+1%/Lv)   |   Stun: 25%
+TP Cost: 36 -&gt; 42 -&gt; 48 -&gt; 54 -&gt; 60 -&gt; 66 -&gt; 72 -&gt; 80 -&gt; 88 -&gt; 96   |   Speed: 1.5x</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -7517,6 +8849,12 @@
           <t>Raise the party's ATK.</t>
         </is>
       </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>ATK: +8% -&gt; +10% -&gt; +12% -&gt; +14% -&gt; +16% (L1-5 Max)
+Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8   |   TP Cost: 12 -&gt; 15 -&gt; 18 -&gt; 20 -&gt; 22   |   Chant: 1.15x</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -7537,6 +8875,12 @@
           <t>Raise the party's DEF.</t>
         </is>
       </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>DEF: +8% -&gt; +10% -&gt; +12% -&gt; +14% -&gt; +16% (L1-5 Max)
+Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8   |   TP Cost: 12 -&gt; 15 -&gt; 18 -&gt; 20 -&gt; 22   |   Chant: 1.15x</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -7557,6 +8901,12 @@
           <t>Create a field that reduces damage for both sides for a time.</t>
         </is>
       </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>Damage reduction: 25% -&gt; 27% -&gt; 29% -&gt; 32% -&gt; 35% (L1-5 Max)
+Turns: 3   |   TP Cost: 28 -&gt; 31 -&gt; 34 -&gt; 37 -&gt; 40   |   Speed: 0.75x   |   Chant: 1.75x</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -7577,6 +8927,12 @@
           <t>Raise encounter rate.</t>
         </is>
       </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>Turns: 10 -&gt; 12 -&gt; 14 -&gt; 16 -&gt; 18 -&gt; 20 -&gt; 22 -&gt; 24 -&gt; 26 -&gt; 28
+TP Cost: 12 -&gt; 11 -&gt; 10 -&gt; 9 -&gt; 8 -&gt; 7 -&gt; 6 -&gt; 5 -&gt; 4 -&gt; 3</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -7597,6 +8953,12 @@
           <t>Sacrifice yourself to revive, heal, and recover status effects for the rest of the party.</t>
         </is>
       </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>Heals RES: 11x -&gt; 13 -&gt; 15 -&gt; 17 -&gt; 19 -&gt; 21 -&gt; 23 -&gt; 25x (L8)
+Recoverable status ailments: 1 (+1/Lv)   |   HP on revival: 10% (+5-10%/Lv) -&gt; 50%</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -7617,6 +8979,12 @@
           <t>Heal an enemy's HP to decrease its physical and magic defense.</t>
         </is>
       </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>DEF: -5% -&gt; -6% -&gt; -7% -&gt; -8% -&gt; -10% (L1-5 Max)   |   Magic defense: -10% -&gt; -15%
+Accuracy: 80% -&gt; 90%   |   HP recovery: 35 -&gt; 25   |   Turns: 3   |   TP: 18 (+2-4/Lv) -&gt; 32</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -7637,6 +9005,12 @@
           <t>Pierce to the back row with a raw magic attack and RES-based extra damage.</t>
         </is>
       </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>Pwr: 100 -&gt; 130 -&gt; 160 -&gt; 200 -&gt; 240 -&gt; 280 -&gt; 320 -&gt; 370 -&gt; 420 -&gt; 480 (L10)
+Accuracy: 80% (+1-2%/Lv) -&gt; 90%   |   TP Cost: 30 (+4/Lv) -&gt; 66   |   Speed: 0.85x</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -7657,6 +9031,12 @@
           <t>Deal enormous damage to one enemy that possesses life. Low chance of instakill.</t>
         </is>
       </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>Pwr: 360 (+40-50/Lv) -&gt; 740   |   Accuracy: 76% (+1%/Lv)   |   Instakill: 12%
+TP Cost: 32 -&gt; 35 -&gt; 38 -&gt; 41 -&gt; 44 -&gt; 47 -&gt; 50 -&gt; 52 -&gt; 54 -&gt; 56   |   Speed: 1.2x</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -7677,6 +9057,12 @@
           <t>Either heal or damage an enemy based on the enemy's HP.</t>
         </is>
       </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>Maximum damage UP   |   Maximum heal UP
+TP Cost: 30 -&gt; 33 -&gt; 36 -&gt; 39 -&gt; 42 (L1-5 Max)   |   Speed: 1.5x   |   Chant: 0.84x -&gt; 0.8x</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -7697,6 +9083,12 @@
           <t>Actual course of action</t>
         </is>
       </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -7717,6 +9109,12 @@
           <t>Actual course of action</t>
         </is>
       </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -7737,6 +9135,12 @@
           <t>Actual course of action</t>
         </is>
       </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -7757,6 +9161,12 @@
           <t>Actual course of action</t>
         </is>
       </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -7777,6 +9187,12 @@
           <t>Actual course of action</t>
         </is>
       </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>dummy
+dummy</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -7797,6 +9213,7 @@
           <t>Deal direct damage back to attacker.</t>
         </is>
       </c>
+      <c r="E242" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -7817,6 +9234,11 @@
           <t>ATK bonus with sword equipped.</t>
         </is>
       </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>ATK bonus: 3% -&gt; 5 -&gt; 7 -&gt; 9 -&gt; 10 -&gt; 11 -&gt; 12 -&gt; 13 -&gt; 14 -&gt; 15% (L10)</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -7837,6 +9259,11 @@
           <t>ATK bonus with axe equipped.</t>
         </is>
       </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>ATK bonus: 3% -&gt; 5 -&gt; 7 -&gt; 9 -&gt; 10 -&gt; 11 -&gt; 12 -&gt; 13 -&gt; 14 -&gt; 15% (L10)</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -7857,6 +9284,11 @@
           <t>ATK bonus with dagger equipped.</t>
         </is>
       </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>ATK bonus: 3% -&gt; 5 -&gt; 7 -&gt; 9 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 15 -&gt; 16 -&gt; 17% (L10)</t>
+        </is>
+      </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -7877,6 +9309,11 @@
           <t>ATK bonus with mace equipped.</t>
         </is>
       </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>ATK bonus: 3% -&gt; 5 -&gt; 7 -&gt; 9 -&gt; 10 -&gt; 11 -&gt; 12 -&gt; 13 -&gt; 14 -&gt; 15% (L10)</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -7897,6 +9334,11 @@
           <t>ATK bonus with lance equipped.</t>
         </is>
       </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>ATK bonus: 3% -&gt; 5 -&gt; 7 -&gt; 9 -&gt; 10 -&gt; 11 -&gt; 12 -&gt; 13 -&gt; 14 -&gt; 15% (L10)</t>
+        </is>
+      </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -7917,6 +9359,11 @@
           <t>ATK bonus with bow equipped.</t>
         </is>
       </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>ATK bonus: 3% -&gt; 5 -&gt; 7 -&gt; 9 -&gt; 10 -&gt; 11 -&gt; 12 -&gt; 13 -&gt; 14 -&gt; 15% (L10)</t>
+        </is>
+      </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -7937,6 +9384,11 @@
           <t>ATK bonus with katana equipped.</t>
         </is>
       </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>ATK bonus: 3% -&gt; 5 -&gt; 7 -&gt; 9 -&gt; 10 -&gt; 11 -&gt; 12 -&gt; 13 -&gt; 14 -&gt; 15% (L10)</t>
+        </is>
+      </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -7957,6 +9409,11 @@
           <t>ATK bonus with projectile weapon equipped.</t>
         </is>
       </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>ATK bonus: 5% -&gt; 7 -&gt; 9 -&gt; 11 -&gt; 13 -&gt; 15 -&gt; 17 -&gt; 18 -&gt; 19 -&gt; 20% (L10)</t>
+        </is>
+      </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -7977,6 +9434,11 @@
           <t>ATK bonus with whip equipped.</t>
         </is>
       </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>ATK bonus: 3% -&gt; 5 -&gt; 7 -&gt; 9 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 15 -&gt; 16 -&gt; 17% (L10)</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -7997,6 +9459,11 @@
           <t>ATK bonus with fan equipped.</t>
         </is>
       </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>ATK bonus: 5% -&gt; 7 -&gt; 9 -&gt; 11 -&gt; 13 -&gt; 15 -&gt; 17 -&gt; 18 -&gt; 19 -&gt; 20% (L10)</t>
+        </is>
+      </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -8017,6 +9484,11 @@
           <t>ATK bonus for all weapons.</t>
         </is>
       </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>ATK bonus: 2% -&gt; 3 -&gt; 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 -&gt; 9 -&gt; 10 -&gt; 12% (L10)</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -8037,6 +9509,11 @@
           <t>Magic attack power bonus.</t>
         </is>
       </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>Magic attack bonus: 6% -&gt; 7 -&gt; 8 -&gt; 9 -&gt; 10 -&gt; 11 -&gt; 12 -&gt; 13 -&gt; 14 -&gt; 15% (L10)</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -8057,6 +9534,12 @@
           <t>Healing magic bonus. Raises healing cap.</t>
         </is>
       </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>HP recovery bonus: 8% -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16 -&gt; 18 -&gt; 20 -&gt; 22 -&gt; 24 -&gt; 26% (L10)
+Heal Cap: +10% -&gt; +20 -&gt; +30 -&gt; +40 -&gt; +50 -&gt; +60 -&gt; +70 -&gt; +80 -&gt; +90 -&gt; +100%</t>
+        </is>
+      </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -8077,6 +9560,11 @@
           <t>Recover HP every turn during battle.</t>
         </is>
       </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>HP recovery: 2% -&gt; 4% -&gt; 6% -&gt; 8% -&gt; 10% (L1-5 Max)</t>
+        </is>
+      </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -8097,6 +9585,11 @@
           <t>Slightly recover HP every turn during battle.</t>
         </is>
       </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>HP recovery: 1% -&gt; 2% -&gt; 3% -&gt; 4% -&gt; 5% (L1-5 Max)</t>
+        </is>
+      </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -8117,6 +9610,11 @@
           <t>Recover TP every turn during battle.</t>
         </is>
       </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>TP recovery: 3 -&gt; 6 -&gt; 9 -&gt; 12 -&gt; 16 (L1-5 Max)</t>
+        </is>
+      </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -8137,6 +9635,11 @@
           <t>Slightly recover TP every turn during battle.</t>
         </is>
       </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>TP recovery: 1 -&gt; 3 -&gt; 5 -&gt; 7 -&gt; 9 (L1-5 Max)</t>
+        </is>
+      </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -8157,6 +9660,11 @@
           <t>Raise resistance to all elements.</t>
         </is>
       </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>Elemental resistance: 6 -&gt; 7 -&gt; 8 -&gt; 9 -&gt; 10 -&gt; 11 -&gt; 12 -&gt; 13 -&gt; 14 -&gt; 15 (L10)</t>
+        </is>
+      </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -8177,6 +9685,11 @@
           <t>Occasionally counterattack after receiving physical damage.</t>
         </is>
       </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>Counterattack rate: 6% -&gt; 9% -&gt; 12% -&gt; 15% -&gt; 18% (L1-5 Max)</t>
+        </is>
+      </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -8197,6 +9710,11 @@
           <t>Occasionally parry and counterattack when targeted by an enemy.</t>
         </is>
       </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>Activation rate: 4% -&gt; 6% -&gt; 8% -&gt; 10% -&gt; 12% (L1-5 Max)</t>
+        </is>
+      </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -8217,6 +9735,11 @@
           <t>Occasionally attack twice when attacking normally.</t>
         </is>
       </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>Double attack rate: 9% -&gt; 12% -&gt; 15% -&gt; 18% -&gt; 21% (L1-5 Max)</t>
+        </is>
+      </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -8237,6 +9760,11 @@
           <t>Occasionally attack thrice when attacking normally.</t>
         </is>
       </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>Triple attack rate: 5% -&gt; 8% -&gt; 11% -&gt; 14% -&gt; 17% (L1-5 Max)</t>
+        </is>
+      </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -8257,6 +9785,11 @@
           <t>Increase evasion rate against stab attacks.</t>
         </is>
       </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>Evasion rate: 20% -&gt; 24% -&gt; 28% -&gt; 32% -&gt; 36% (L1-5 Max)</t>
+        </is>
+      </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -8277,6 +9810,11 @@
           <t>Occasionally parry when receiving long-range attacks.</t>
         </is>
       </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>Activation rate: 10% -&gt; 15% -&gt; 20% -&gt; 25% -&gt; 30% (L1-5 Max)</t>
+        </is>
+      </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -8297,6 +9835,11 @@
           <t>Occasionally survive at 1 HP after being dealt fatal damage.</t>
         </is>
       </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>Survival rate: 10% -&gt; 15% -&gt; 20% -&gt; 25% -&gt; 30% (L1-5 Max)</t>
+        </is>
+      </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -8317,6 +9860,11 @@
           <t>Occasionally Defend automatically when receiving physical attacks.</t>
         </is>
       </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>Auto-guard rate: 4% -&gt; 6% -&gt; 8% -&gt; 10% -&gt; 12% (L1-5 Max)</t>
+        </is>
+      </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -8337,6 +9885,11 @@
           <t>Can equip two one-handed weapons at the same time.</t>
         </is>
       </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>Sub-weapon ATK: 30% -&gt; 35 -&gt; 40 -&gt; 45 -&gt; 50 -&gt; 54 -&gt; 58 -&gt; 62 -&gt; 68 -&gt; 72% (L10)</t>
+        </is>
+      </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -8357,6 +9910,11 @@
           <t>Convert some received damage to TP.</t>
         </is>
       </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>TP conversion: 4% -&gt; 8% -&gt; 12% -&gt; 16% -&gt; 20% (L1-5 Max)</t>
+        </is>
+      </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -8377,6 +9935,11 @@
           <t>Occasionally instakill when inflicting a critical hit.</t>
         </is>
       </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>Activation rate: 8% -&gt; 11% -&gt; 14% -&gt; 17% -&gt; 20% (L1-5 Max)</t>
+        </is>
+      </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -8397,6 +9960,11 @@
           <t>With bow equipped, occasionally halt an enemy's action.</t>
         </is>
       </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>Activation rate: 2% -&gt; 3% -&gt; 4% -&gt; 5% -&gt; 6% (L1-5 Max)</t>
+        </is>
+      </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -8417,6 +9985,11 @@
           <t>With bow equipped, occasionally attack again after an ally's attack.</t>
         </is>
       </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>Activation rate: 4% -&gt; 6% -&gt; 8% -&gt; 10% -&gt; 12% (L1-5 Max)</t>
+        </is>
+      </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -8437,6 +10010,11 @@
           <t>Gain increased speed based on missing HP.</t>
         </is>
       </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>Speed increase: 15% -&gt; 16% -&gt; 17% -&gt; 18% -&gt; 20% (L1-5 Max)</t>
+        </is>
+      </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -8457,6 +10035,11 @@
           <t>Debuff an enemy when they inflict short-range damage.</t>
         </is>
       </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>Number of possible debuffs: 1 -&gt; 2 -&gt; 3 -&gt; 4 -&gt; 5 -&gt; 6 (L6)</t>
+        </is>
+      </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -8477,6 +10060,11 @@
           <t>Increase ATK while inflicted with status ailments.</t>
         </is>
       </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>ATK: +15% -&gt; +18% -&gt; +21% -&gt; +24% -&gt; +27% (L1-5 Max)</t>
+        </is>
+      </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -8497,6 +10085,7 @@
           <t>Nullify the effects of enemy Dark Auras.</t>
         </is>
       </c>
+      <c r="E277" t="inlineStr"/>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -8517,6 +10106,7 @@
           <t>No longer suffer counterattacks from enemies.</t>
         </is>
       </c>
+      <c r="E278" t="inlineStr"/>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -8537,6 +10127,11 @@
           <t>Decrease physical damage to the back row when using a shield in the front row.</t>
         </is>
       </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>Physical damage: -6% -&gt; -7% -&gt; -8% -&gt; -9% -&gt; -10% (L1-5 Max)</t>
+        </is>
+      </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -8557,6 +10152,11 @@
           <t>Occasionally nullify physical damage.</t>
         </is>
       </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>Activation rate: 8% -&gt; 9% -&gt; 10% -&gt; 11% -&gt; 12% (L1-5 Max)</t>
+        </is>
+      </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -8577,6 +10177,11 @@
           <t>Automatically heal inflicted status ailments at the start of each turn.</t>
         </is>
       </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>LvUp: Can cure poison &gt; paralysis &gt; silence &gt; freeze &gt; sleep &gt; slow</t>
+        </is>
+      </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
@@ -8597,6 +10202,11 @@
           <t>Briefly increase ATK and DEX when HP drops below 50%.</t>
         </is>
       </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>ATK/DEX: +10% -&gt; +11% -&gt; +12% -&gt; +13% -&gt; +15% (L1-5 Max)</t>
+        </is>
+      </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -8617,6 +10227,11 @@
           <t>Make it harder for chants, songs, and dances to be interrupted.</t>
         </is>
       </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>LvUp: Interruption rate DOWN</t>
+        </is>
+      </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -8637,6 +10252,11 @@
           <t>Reduce chant time.</t>
         </is>
       </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>Chant time: -8% -&gt; -11% -&gt; -14% -&gt; -17% -&gt; -20% (L1-5 Max)</t>
+        </is>
+      </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
@@ -8657,6 +10277,11 @@
           <t>Reduce TP Cost in battle.</t>
         </is>
       </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>TP Cost reduction: 10% -&gt; 15% -&gt; 20% -&gt; 25% -&gt; 30% (L1-5 Max)</t>
+        </is>
+      </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
@@ -8677,6 +10302,11 @@
           <t>Heighten magic accuracy.</t>
         </is>
       </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>Accuracy: 3% -&gt; 5% -&gt; 7% -&gt; 9% -&gt; 12% (L1-5 Max)</t>
+        </is>
+      </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -8697,6 +10327,11 @@
           <t>Limit enemies' preemptive attacks.</t>
         </is>
       </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>Enemy preemptive attack rate: -20% -&gt; -28% -&gt; -36% -&gt; -44% -&gt; -50% (L1-5 Max)</t>
+        </is>
+      </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
@@ -8717,6 +10352,11 @@
           <t>Increase party's preemptive attack rate.</t>
         </is>
       </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>Preemptive attack rate: 8% -&gt; 11% -&gt; 14% -&gt; 17% -&gt; 20% (L1-5 Max)</t>
+        </is>
+      </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
@@ -8737,6 +10377,11 @@
           <t>May escape from battle more easily.</t>
         </is>
       </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>Battle escape rate: 20% -&gt; 25% -&gt; 30% -&gt; 35% -&gt; 40% (L1-5 Max)</t>
+        </is>
+      </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -8757,6 +10402,11 @@
           <t>Increase the enemies' item drop rate.</t>
         </is>
       </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>Item drop rate: 4% -&gt; 6% -&gt; 8% -&gt; 10% -&gt; 12% (L1-5 Max)</t>
+        </is>
+      </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
@@ -8777,6 +10427,11 @@
           <t>Increase the amount of money the enemies drop.</t>
         </is>
       </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>Gold drop rate: 25% -&gt; 50% -&gt; 75% -&gt; 100% -&gt; 125% (L1-5 Max)</t>
+        </is>
+      </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
@@ -8797,6 +10452,11 @@
           <t>Sometimes pick up items while moving around the dungeons.</t>
         </is>
       </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>Found item quality: 1 -&gt; 2 -&gt; 3 -&gt; 4 -&gt; 5 (L1-5 Max)</t>
+        </is>
+      </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
@@ -8817,6 +10477,12 @@
           <t>Party's HP and TP is restored slightly after a battle.</t>
         </is>
       </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>Post-battle HP: 6% -&gt; 7% -&gt; 8% -&gt; 10% -&gt; 12% (L1-5 Max)
+Post-battle TP: 3% -&gt; 4% -&gt; 5% -&gt; 7% -&gt; 9%</t>
+        </is>
+      </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -8837,6 +10503,11 @@
           <t>Occasionally keep disposable items after using them in battle.</t>
         </is>
       </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>Item keep rate: 25% -&gt; 27% -&gt; 29% -&gt; 32% -&gt; 35% (L1-5 Max)</t>
+        </is>
+      </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -8857,6 +10528,11 @@
           <t>Increase the effects of HP and TP recovery items during battle.</t>
         </is>
       </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>Item effects: 10% -&gt; 20 -&gt; 30 -&gt; 40 -&gt; 50 -&gt; 60 -&gt; 70 -&gt; 80 -&gt; 90 -&gt; 100% (L10)</t>
+        </is>
+      </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -8877,6 +10553,11 @@
           <t>Become capable of performing two songs at once.</t>
         </is>
       </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>Speed: 6% -&gt; 9% -&gt; 12% -&gt; 15% -&gt; 18% (L1-5 Max)</t>
+        </is>
+      </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -8897,6 +10578,11 @@
           <t>Become capable of performing two dances at once.</t>
         </is>
       </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>Speed: 6% -&gt; 9% -&gt; 12% -&gt; 15% -&gt; 18% (L1-5 Max)</t>
+        </is>
+      </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
@@ -8917,6 +10603,11 @@
           <t>Become capable of controlling two dolls at once.</t>
         </is>
       </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>Speed: 6% -&gt; 9% -&gt; 12% -&gt; 15% -&gt; 18% (L1-5 Max)</t>
+        </is>
+      </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
@@ -8937,6 +10628,11 @@
           <t>Increase doll power with the strength of the equipped Sealbook.</t>
         </is>
       </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>Sealbook ability: +15% -&gt; +18% -&gt; +21% -&gt; +24% -&gt; +27% (L1-5 Max)</t>
+        </is>
+      </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -8957,6 +10653,11 @@
           <t>Increased effects for all maid skills.</t>
         </is>
       </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>Maid skill bonus: 1% -&gt; 2 -&gt; 3 -&gt; 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 -&gt; 9 -&gt; 10% (L10)</t>
+        </is>
+      </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -8977,6 +10678,11 @@
           <t>Increased effects for all songs.</t>
         </is>
       </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>Singing skill bonus: 3% -&gt; 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 -&gt; 9 -&gt; 10 -&gt; 11 -&gt; 12% (L10)</t>
+        </is>
+      </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
@@ -8997,6 +10703,11 @@
           <t>Increased effects for all dances.</t>
         </is>
       </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>Dancing skill bonus: 3% -&gt; 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 -&gt; 9 -&gt; 10 -&gt; 11 -&gt; 12% (L10)</t>
+        </is>
+      </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
@@ -9017,6 +10728,11 @@
           <t>Increased effects for all doll skills.</t>
         </is>
       </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>Doll skill bonus: 3% -&gt; 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 -&gt; 9 -&gt; 10 -&gt; 11 -&gt; 12% (L10)</t>
+        </is>
+      </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
@@ -9037,6 +10753,11 @@
           <t>Occasionally attack twice when attacking normally.</t>
         </is>
       </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>Double attack rate: 20% -&gt; 21 -&gt; 22 -&gt; 23 -&gt; 24 -&gt; 25 -&gt; 26 -&gt; 28 -&gt; 30 -&gt; 32% (L10)</t>
+        </is>
+      </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
@@ -9057,6 +10778,11 @@
           <t>Reduce chant time for songs.</t>
         </is>
       </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>Song chant time: -10% -&gt; -11 -&gt; -12 -&gt; -13 -&gt; -14 -&gt; -15 -&gt; -16 -&gt; -17 -&gt; -18 -&gt; -20%</t>
+        </is>
+      </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
@@ -9077,6 +10803,11 @@
           <t>Reduce purchase and identification prices at shops.</t>
         </is>
       </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>Negotiation rate: 10% -&gt; 14% -&gt; 18% -&gt; 22% -&gt; 25% (L1-5 Max)</t>
+        </is>
+      </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -9097,6 +10828,11 @@
           <t>Mesmerize enemies, causing them to occasionally do nothing.</t>
         </is>
       </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>Occurrence rate: 3% -&gt; 4% -&gt; 5% -&gt; 6% -&gt; 7% (L1-5 Max)</t>
+        </is>
+      </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
@@ -9117,6 +10853,7 @@
           <t>Nullify first hit of battle against user (does not work for status ailments).</t>
         </is>
       </c>
+      <c r="E308" t="inlineStr"/>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
@@ -9137,6 +10874,7 @@
           <t>Heighten the probability of beneficial results for random effect skills.</t>
         </is>
       </c>
+      <c r="E309" t="inlineStr"/>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
@@ -9157,6 +10895,7 @@
           <t>Whip skill. Strike back with a normal attack before a targeted attack hits you.</t>
         </is>
       </c>
+      <c r="E310" t="inlineStr"/>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
@@ -9177,6 +10916,7 @@
           <t>Occasionally get the first action regardless of speed.</t>
         </is>
       </c>
+      <c r="E311" t="inlineStr"/>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
@@ -9197,6 +10937,7 @@
           <t>Occasionally land critical hits with offensive spells.</t>
         </is>
       </c>
+      <c r="E312" t="inlineStr"/>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
@@ -9217,6 +10958,7 @@
           <t>Increase doll summon duration by 1 turn.</t>
         </is>
       </c>
+      <c r="E313" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs: add equipment and enchantments guide sections
</commit_message>
<xml_diff>
--- a/data_tables/guide_text.xlsx
+++ b/data_tables/guide_text.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -491,153 +491,187 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>equip_section</t>
+          <t>enchantments_title</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>#### Usable Equipment</t>
+          <t># Equipment Enchantments</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Equipment compatibility based on class usability flags.</t>
+          <t>Reference for equipment enchantments, scaling per equipped piece, stacking rules, and caps verified in the game engine.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>formulas_title</t>
+          <t>equip_section</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t># Battle Formulas</t>
+          <t>#### Usable Equipment</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Reference for combat mathematics, damage functions, turn order calculations, and status ailment checks in Dungeon Travelers 2-2. Every formula represents the exact logic executed by the game engine.</t>
+          <t>Equipment compatibility based on class usability flags.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>growth_section</t>
+          <t>equipment_title</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>#### Stat Growth</t>
+          <t># Equipment</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Reference for weapons, armor, accessories, weapon recovery delay ranks, and equipment upgrade rates in Dungeon Travelers 2-2.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>modifier_section</t>
+          <t>formulas_title</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>#### Weapon Specialty Modifiers</t>
+          <t># Battle Formulas</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Equipping a specialized weapon, shield, or accessory grants a percentage bonus to all non-zero stats on that piece: `int((character_stat + piece_stat) * modifier)`.</t>
+          <t>Reference for combat mathematics, damage functions, turn order calculations, and status ailment checks in Dungeon Travelers 2-2. Every formula represents the exact logic executed by the game engine.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>overview_section</t>
+          <t>growth_section</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>#### Class Overview</t>
+          <t>#### Stat Growth</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>readme_glossary</t>
+          <t>modifier_section</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>## Glossary</t>
+          <t>#### Weapon Specialty Modifiers</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Core combat parameters, calculations, and mechanical terms used throughout this guide.</t>
+          <t>Equipping a specialized weapon, shield, or accessory grants a percentage bonus to all non-zero stats on that piece: `int((character_stat + piece_stat) * modifier)`.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>readme_how_to_read</t>
+          <t>overview_section</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>## How to Read the Tables</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Stat tables record raw class attributes at milestone levels from 1 to 99. Modifiers operate additively unless specified by game logic. Equipment usability lists weapon classes and defensive gear categories supported by internal compatibility bitmasks.</t>
+          <t>#### Class Overview</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>readme_title</t>
+          <t>readme_glossary</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t># Dungeon Travelers 2-2 Reference Guide (Vanilla)</t>
+          <t>## Glossary</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Player reference documentation for the original English PC release of Dungeon Travelers 2-2. All data, mechanics, and formulas are compiled directly from the original game files.</t>
+          <t>Core combat parameters, calculations, and mechanical terms used throughout this guide.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>skills_section</t>
+          <t>readme_how_to_read</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>#### Learned Skills</t>
+          <t>## How to Read the Tables</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Stat tables record raw class attributes at milestone levels from 1 to 99. Modifiers operate additively unless specified by game logic. Equipment usability lists weapon classes and defensive gear categories supported by internal compatibility bitmasks.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>readme_title</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t># Dungeon Travelers 2-2 Reference Guide (Vanilla)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Player reference documentation for the original English PC release of Dungeon Travelers 2-2. All data, mechanics, and formulas are compiled directly from the original game files.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>skills_section</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>#### Learned Skills</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>skills_title</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t># Skills</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>Reference for all skills learned by player classes, including category, TP and SP costs, action speed, cast speed, target, range, and exact numerical scaling across all levels.</t>
         </is>
@@ -654,7 +688,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B42"/>
+  <dimension ref="A1:B57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -672,490 +706,670 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>agi</t>
+          <t>accessory</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>AGI</t>
+          <t>Accessory</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>atk</t>
+          <t>agi</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ATK</t>
+          <t>AGI</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>base_class</t>
+          <t>armor</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Base Class</t>
+          <t>Armor</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>bonus</t>
+          <t>atk</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Modifier</t>
+          <t>ATK</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>cast_factor</t>
+          <t>base_class</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Chant Speed</t>
+          <t>Base Class</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>category</t>
+          <t>body_armor</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>Body Armor</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>character</t>
+          <t>bonus</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Character</t>
+          <t>Modifier</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>classes</t>
+          <t>cap</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Classes</t>
+          <t>Cap / Limit</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>cast_factor</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Count</t>
+          <t>Chant Speed</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>def</t>
+          <t>category</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>DEF</t>
+          <t>Type</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>character</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Effect &amp; Scaling</t>
+          <t>Character</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>dex</t>
+          <t>classes</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>DEX</t>
+          <t>Classes</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>equipment_type</t>
+          <t>count</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Equipment Type</t>
+          <t>Count</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>gear_categories</t>
+          <t>def</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Defensive Gear</t>
+          <t>DEF</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>hp</t>
+          <t>delay_mult</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Delay Mult</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>delay_rank</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>Delay Rank</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>join_point</t>
+          <t>description</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Join Point</t>
+          <t>Effect &amp; Scaling</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dex</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Level</t>
+          <t>DEX</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>line</t>
+          <t>enchantment</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Line</t>
+          <t>Enchantment</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>max_lv</t>
+          <t>equipment_type</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Max Lv</t>
+          <t>Equipment Type</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>overview</t>
+          <t>gear_categories</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Class Overview</t>
+          <t>Defensive Gear</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>profile</t>
+          <t>headgear</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Combat Role &amp; Profile</t>
+          <t>Headgear</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>range</t>
+          <t>hp</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Range</t>
+          <t>HP</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>rank</t>
+          <t>innate_enchants</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Rank</t>
+          <t>Innate Enchants</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ranks</t>
+          <t>int</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Rank Scaling</t>
+          <t>INT</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>res</t>
+          <t>join_point</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>RES</t>
+          <t>Join Point</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>route</t>
+          <t>level</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Promotion Route</t>
+          <t>Level</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>skill</t>
+          <t>line</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Skill</t>
+          <t>Line</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>slot</t>
+          <t>magnitude</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Slot</t>
+          <t>Value / Scaling</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>sp_cost</t>
+          <t>max_lv</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Total SP</t>
+          <t>Max Lv</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>speed_factor</t>
+          <t>overview</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Action Speed</t>
+          <t>Class Overview</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>start_exp</t>
+          <t>profile</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Starting EXP</t>
+          <t>Combat Role &amp; Profile</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>start_level</t>
+          <t>range</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Starting Lv</t>
+          <t>Range</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>target</t>
+          <t>rank</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Target</t>
+          <t>Rank</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>tier</t>
+          <t>ranks</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Tier</t>
+          <t>Rank Scaling</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>tp</t>
+          <t>res</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>RES</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>tp_cost</t>
+          <t>route</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>TP Cost</t>
+          <t>Promotion Route</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>turns</t>
+          <t>shield</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Duration</t>
+          <t>Shield</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>unique_skill</t>
+          <t>skill</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Unique Skill</t>
+          <t>Skill</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>value</t>
+          <t>slot</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Value</t>
+          <t>Slot</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
+          <t>sp_cost</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Total SP</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>speed_factor</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Action Speed</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>stacking</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Stacking Rule</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>start_exp</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Starting EXP</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>start_level</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Starting Lv</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>tier</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>tp</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>tp_cost</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>TP Cost</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>turns</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Duration</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>two_handed</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>2-Handed</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>unique_skill</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Unique Skill</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>upgrade_rate</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Upgrade Rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>weapon</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Weapon</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
           <t>weapon_types</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B57" t="inlineStr">
         <is>
           <t>Weapon Types</t>
         </is>

</xml_diff>

<commit_message>
docs: add enemies, bosses, summons, mercenaries, and progression
</commit_message>
<xml_diff>
--- a/data_tables/guide_text.xlsx
+++ b/data_tables/guide_text.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -674,6 +674,91 @@
       <c r="C16" t="inlineStr">
         <is>
           <t>Reference for all skills learned by player classes, including category, TP and SP costs, action speed, cast speed, target, range, and exact numerical scaling across all levels.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>enemies_title</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t># Enemies</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Catalog of all enemies in Dungeon Travelers 2-2 organized by habitat, including combat stats, element resistances, ailment immunities, attack skills, and drop rates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>bosses_title</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t># Boss Encounters</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Reference for fixed story and postgame boss encounters, including combat stats, elemental resistances, attack repertoires, and complete AI behavior scripts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>summons_title</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t># Grand Sealbook Summons</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Reference for all 35 Grand Sealbook summons, detailing stat growth factors, attack repertoires, AI weights, and passive enchantments across all three forms.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>mercenaries_title</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t># Mercenaries (Guest Allies)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Reference for all hireable mercenaries at the Tavern, including unlock requirements, hiring costs, contract lengths, growth stages, combat stats, attack repertoires, and AI scripts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>progression_title</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t># Game Progression</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Experience and skill point curves from Level 1 to 99, crown reset stat bonus milestones, and encounter level ranges across all dungeon floors.</t>
         </is>
       </c>
     </row>
@@ -688,7 +773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B57"/>
+  <dimension ref="A1:B96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1372,6 +1457,474 @@
       <c r="B57" t="inlineStr">
         <is>
           <t>Weapon Types</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>exp</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>EXP</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>race</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Race</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>resistances</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Resistances</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>immunities</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Immunities</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>drops</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Item Drops</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>equip_drop</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Equipment Drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>snack</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>steal</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Steal</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>attacks</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Attacks</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>passives</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Passives</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>ai_script</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>AI Behavior</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>opening</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Opening Actions</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>action_sets</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Action Sets</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>slash</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Slash</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>stab</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Stab</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>bash</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Bash</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>fire</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Fire</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>water</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Water</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>wind</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Wind</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>earth</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Earth</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>lightning</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Lightning</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>power</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Power</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>speed</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>cost</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>contract</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>unlock</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Unlock Point</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>stage</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Stage</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>factors</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Stat Multipliers</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>req_exp</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Required EXP</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>total_exp</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Cumulative EXP</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>sp_gain</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>SP Gained</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>dungeon</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Dungeon</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>floor</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Floor</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>enemy_levels</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Random Enemy Levels</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>boss_levels</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Boss Encounters</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>bonus_stats</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Bonus Stats</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>reset_level</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Reset Level</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>cap_info</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Stat Cap</t>
         </is>
       </c>
     </row>

</xml_diff>